<commit_message>
Deliverables rename, yy position, fix template tokens, all 6 languages
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mac/GitHub Repos/GKIMWebsite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FEF55A3-2FE8-A149-94E0-DD56C40FC364}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0713BD9E-9834-5A4A-8879-02E6FA704A6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="44800" windowHeight="24700" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -492,10 +492,10 @@
     <t>nav.link.outputs</t>
   </si>
   <si>
-    <t>Outputs</t>
-  </si>
-  <si>
-    <t>Ergebnisse</t>
+    <t>Deliverables</t>
+  </si>
+  <si>
+    <t>Liefergegenstände</t>
   </si>
   <si>
     <t>Livrables</t>
@@ -504,7 +504,7 @@
     <t>Resultaten</t>
   </si>
   <si>
-    <t>成果</t>
+    <t>交付物</t>
   </si>
   <si>
     <t>Kết quả</t>
@@ -1296,22 +1296,22 @@
     <t>Step 3 title</t>
   </si>
   <si>
-    <t>Deliver — Build-Ready Outputs</t>
-  </si>
-  <si>
-    <t>Liefern — Baufertige Ergebnisse</t>
-  </si>
-  <si>
-    <t>Livrer — Des livrables prêts à construire</t>
-  </si>
-  <si>
-    <t>Opleveren — Bouwklare resultaten</t>
-  </si>
-  <si>
-    <t>交付——可构建的成果</t>
-  </si>
-  <si>
-    <t>Bàn giao — Kết quả sẵn sàng để xây dựng</t>
+    <t>Deliver — Design Deliverables</t>
+  </si>
+  <si>
+    <t>Liefern — Design-Liefergegenstände</t>
+  </si>
+  <si>
+    <t>Livrer — Livrables de conception</t>
+  </si>
+  <si>
+    <t>Opleveren — Ontwerpresultaten</t>
+  </si>
+  <si>
+    <t>交付——设计交付物</t>
+  </si>
+  <si>
+    <t>Bàn giao — Kết quả thiết kế</t>
   </si>
   <si>
     <t>gears.kl</t>
@@ -1395,49 +1395,49 @@
     <t>outputs</t>
   </si>
   <si>
-    <t>What You Actually Get</t>
-  </si>
-  <si>
-    <t>Was Sie tatsächlich erhalten</t>
-  </si>
-  <si>
-    <t>Ce que vous obtenez réellement</t>
-  </si>
-  <si>
-    <t>Wat u daadwerkelijk krijgt</t>
-  </si>
-  <si>
-    <t>您实际获得的内容</t>
-  </si>
-  <si>
-    <t>Những gì bạn thực sự nhận được</t>
+    <t>Design Deliverables</t>
+  </si>
+  <si>
+    <t>Design-Liefergegenstände</t>
+  </si>
+  <si>
+    <t>Livrables de conception</t>
+  </si>
+  <si>
+    <t>Ontwerpresultaten</t>
+  </si>
+  <si>
+    <t>设计交付物</t>
+  </si>
+  <si>
+    <t>Kết quả thiết kế</t>
   </si>
   <si>
     <t>outputs.h</t>
   </si>
   <si>
     <t>Not advisory.
-Production.</t>
+Deliverables.</t>
   </si>
   <si>
     <t>Keine Beratung.
-Produktion.</t>
+Liefergegenstände.</t>
   </si>
   <si>
     <t>Pas de conseil.
-De la production.</t>
+Des livrables.</t>
   </si>
   <si>
     <t>Geen advies.
-Productie.</t>
+Liefergegenstanden.</t>
   </si>
   <si>
     <t>不是咨询。
-而是交付。</t>
+而是交付物。</t>
   </si>
   <si>
     <t>Không phải tư vấn.
-Mà là sản xuất.</t>
+Mà là kết quả bàn giao.</t>
   </si>
   <si>
     <t>outputs.intro.p1</t>
@@ -1494,10 +1494,10 @@
     <t>Output 01 label</t>
   </si>
   <si>
-    <t>Output 01 — Capability Map</t>
-  </si>
-  <si>
-    <t>Ergebnis 01 — Fähigkeitskarte</t>
+    <t>Deliverable 01 — Capability Map</t>
+  </si>
+  <si>
+    <t>Liefergegenstand 01 — Fähigkeitskarte</t>
   </si>
   <si>
     <t>Livrable 01 — Cartographie des capacités</t>
@@ -1506,7 +1506,7 @@
     <t>Resultaat 01 — Capaciteitskaart</t>
   </si>
   <si>
-    <t>成果01——能力图谱</t>
+    <t>交付物01——能力图谱</t>
   </si>
   <si>
     <t>Kết quả 01 — Bản đồ năng lực</t>
@@ -1542,10 +1542,10 @@
     <t>Output 02 label</t>
   </si>
   <si>
-    <t>Output 02 — Workflow Architecture</t>
-  </si>
-  <si>
-    <t>Ergebnis 02 — Workflow-Architektur</t>
+    <t>Deliverable 02 — Workflow Architecture</t>
+  </si>
+  <si>
+    <t>Liefergegenstand 02 — Workflow-Architektur</t>
   </si>
   <si>
     <t>Livrable 02 — Architecture des flux de travail</t>
@@ -1554,7 +1554,7 @@
     <t>Resultaat 02 — Workflowarchitectuur</t>
   </si>
   <si>
-    <t>成果02——工作流架构</t>
+    <t>交付物02——工作流架构</t>
   </si>
   <si>
     <t>Kết quả 02 — Kiến trúc quy trình làm việc</t>

</xml_diff>

<commit_message>
Translate papers section; wire all card strings to spreadsheet
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -1452,7 +1452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J125"/>
+  <dimension ref="A1:J144"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="11" min="1" max="1"/>
@@ -6900,6 +6900,692 @@
       <c r="J125" t="inlineStr">
         <is>
           <t>en</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>papers.title</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Go-deeper bridge section heading</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>GKIM Papers —
+Original thinking on
+AI-native business design</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>GKIM Papers —
+Originäres Denken über
+KI-native Geschäftsmodelle</t>
+        </is>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>GKIM Papers —
+Tư duy độc lập về
+thiết kế kinh doanh theo hướng AI</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>GKIM Papers —
+Original thinking on
+AI-native business design</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>papers.sub</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>Fifteen papers across five themes. Written for founders, operators, and investors who want to understand the architecture of what's coming.</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Fünfzehn Papiere über fünf Themen. Geschrieben für Gründer, Operatoren und Investoren, die die Architektur der kommenden Entwicklungen verstehen möchten.</t>
+        </is>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>Mười lăm bài viết trên năm chủ đề. Viết cho các nhà sáng lập, những người điều hành và nhà đầu tư muốn hiểu rõ kiến trúc của những gì sắp tới.</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>Fifteen papers across five themes. Written for founders, operators, and investors who want to understand the architecture of what's coming.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>papers.s1.section</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Category label</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>Foundations</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Grundlagen</t>
+        </is>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>Nền tảng</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>Foundations</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>papers.s1.name</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Category subtitle</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>What is an AI-Native Business?</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Was ist ein KI-natives Geschäftsmodell?</t>
+        </is>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>Kinh doanh theo hướng AI là gì?</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>What is an AI-Native Business?</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>papers.s1.count</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Paper count label</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>3 Papiere</t>
+        </is>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>3 bài viết</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>papers.s2.section</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Category label</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>The Case For</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Das Argument dafür</t>
+        </is>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Lý do để tin tưởng</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>The Case For</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>papers.s2.name</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Category subtitle</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>The Strategic &amp; Economic Argument</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Das strategische und ökonomische Argument</t>
+        </is>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Lập luận chiến lược và kinh tế</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>The Strategic &amp; Economic Argument</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>papers.s2.count</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>3 Papiere</t>
+        </is>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>3 bài viết</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>papers.s3.section</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Category label</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>Trust &amp; Safety</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Vertrauen und Sicherheit</t>
+        </is>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>Tin tưởng &amp; An toàn</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>Trust &amp; Safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>papers.s3.name</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Category subtitle</t>
+        </is>
+      </c>
+      <c r="D135" t="inlineStr">
+        <is>
+          <t>Governance, Humans &amp; Accountability</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>Governance, Menschen und Verantwortung</t>
+        </is>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>Quản lý, Con người &amp; Trách nhiệm</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>Governance, Humans &amp; Accountability</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>papers.s3.count</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>3 Papiere</t>
+        </is>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>3 bài viết</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>papers.s4.section</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Category label</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>Founder's Playbook</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>Playbook für Gründer</t>
+        </is>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>Sổ tay nhà sáng lập</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>Founder's Playbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>papers.s4.name</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Category subtitle</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Practical Conviction for Builders</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Praktische Überzeugung für Builder</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Quyết tâm thực tiễn cho những người xây dựng</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>Practical Conviction for Builders</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>papers.s4.count</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>3 Papiere</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>3 bài viết</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>papers.s5.section</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Category label</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>Architecture &amp; Lifecycle</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Architektur und Lebenszyklus</t>
+        </is>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>Kiến trúc &amp; Vòng đời</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>Architecture &amp; Lifecycle</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>papers.s5.name</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Category subtitle</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>How These Businesses Are Built</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>Wie diese Geschäftsmodelle aufgebaut sind</t>
+        </is>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>Cách các doanh nghiệp này được xây dựng</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>How These Businesses Are Built</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>papers.s5.count</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>3 Papiere</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>3 bài viết</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>papers.foot</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Footer note</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Each paper is 7–11 minutes. Full PDFs coming soon. Written from Cambridge — not from a conference stage.</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Jedes Papier dauert 7–11 Minuten zum Lesen. Vollständige PDFs folgen in Kürze. Geschrieben aus Cambridge — nicht von einer Konferenzbühne.</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Mỗi bài viết mất 7–11 phút để đọc. Toàn bộ PDF sẽ ra mắt sớm. Viết từ Cambridge — không phải từ một sân khấu hội thảo.</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>Each paper is 7–11 minutes. Full PDFs coming soon. Written from Cambridge — not from a conference stage.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>papers.cta</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>papers</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>CTA link text</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Read GKIM Papers →</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>GKIM Papers lesen →</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Đọc GKIM Papers →</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>Read GKIM Papers →</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add flag emojis to language switcher
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -820,7 +820,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="11" min="1" max="1"/>
@@ -871,6 +871,11 @@
           <t>notes</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>flag</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="36" customHeight="1" s="11">
       <c r="A2" s="2" t="inlineStr">
@@ -913,6 +918,11 @@
           <t>Canonical — default. Global audience. Current site copy.</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>🇬🇧</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="36" customHeight="1" s="11">
       <c r="A3" s="2" t="inlineStr">
@@ -955,6 +965,11 @@
           <t>Priority European market. Emphasis on rigour, methodology, enterprise credibility.</t>
         </is>
       </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>🇩🇪</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="36" customHeight="1" s="11">
       <c r="A4" s="2" t="inlineStr">
@@ -997,6 +1012,11 @@
           <t>Strategic framing, intellectual positioning. Paris/Brussels audience.</t>
         </is>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>🇫🇷</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="36" customHeight="1" s="11">
       <c r="A5" s="2" t="inlineStr">
@@ -1039,6 +1059,11 @@
           <t>Commercial directness. Amsterdam/Rotterdam tech and VC audience.</t>
         </is>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>🇳🇱</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="36" customHeight="1" s="11">
       <c r="A6" s="2" t="inlineStr">
@@ -1081,6 +1106,11 @@
           <t>Systems thinking, enterprise value, Cambridge credibility. APAC enterprise.</t>
         </is>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>🇨🇳</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="36" customHeight="1" s="11">
       <c r="A7" s="2" t="inlineStr">
@@ -1121,6 +1151,11 @@
       <c r="H7" s="2" t="inlineStr">
         <is>
           <t>HCMC office presence, regional expertise, founder story. Vietnam market.</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>🇻🇳</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
rebuild: revert draft languages, flags live
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -164,13 +164,13 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -539,18 +539,18 @@
   <dimension ref="A1:B26"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" style="11" min="1" max="1"/>
-    <col width="80" customWidth="1" style="11" min="2" max="2"/>
+    <col width="22" customWidth="1" style="12" min="1" max="1"/>
+    <col width="80" customWidth="1" style="12" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" s="11">
-      <c r="A1" s="10" t="inlineStr">
+    <row r="1" ht="28" customHeight="1" s="12">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>GKIM Digital — Multilingual Content Workbook</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="30" customHeight="1" s="11">
+    <row r="2" ht="30" customHeight="1" s="12">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -562,11 +562,11 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="18" customHeight="1" s="11">
+    <row r="3" ht="18" customHeight="1" s="12">
       <c r="A3" s="3" t="n"/>
       <c r="B3" s="2" t="n"/>
     </row>
-    <row r="4" ht="18" customHeight="1" s="11">
+    <row r="4" ht="18" customHeight="1" s="12">
       <c r="A4" s="1" t="inlineStr">
         <is>
           <t>SHEETS</t>
@@ -574,7 +574,7 @@
       </c>
       <c r="B4" s="2" t="n"/>
     </row>
-    <row r="5" ht="18" customHeight="1" s="11">
+    <row r="5" ht="18" customHeight="1" s="12">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>1. README</t>
@@ -586,7 +586,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="30" customHeight="1" s="11">
+    <row r="6" ht="30" customHeight="1" s="12">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>2. languages</t>
@@ -598,7 +598,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="30" customHeight="1" s="11">
+    <row r="7" ht="30" customHeight="1" s="12">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>3. strategic_emphasis</t>
@@ -610,7 +610,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1" s="11">
+    <row r="8" ht="30" customHeight="1" s="12">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>4. strings</t>
@@ -622,7 +622,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1" s="11">
+    <row r="9" ht="30" customHeight="1" s="12">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>5. meta_seo</t>
@@ -634,7 +634,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="30" customHeight="1" s="11">
+    <row r="10" ht="30" customHeight="1" s="12">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>6. config</t>
@@ -646,11 +646,11 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" s="11">
+    <row r="11" ht="18" customHeight="1" s="12">
       <c r="A11" s="3" t="n"/>
       <c r="B11" s="2" t="n"/>
     </row>
-    <row r="12" ht="18" customHeight="1" s="11">
+    <row r="12" ht="18" customHeight="1" s="12">
       <c r="A12" s="1" t="inlineStr">
         <is>
           <t>HOW TO USE</t>
@@ -658,7 +658,7 @@
       </c>
       <c r="B12" s="2" t="n"/>
     </row>
-    <row r="13" ht="30" customHeight="1" s="11">
+    <row r="13" ht="30" customHeight="1" s="12">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Step 1</t>
@@ -670,7 +670,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="30" customHeight="1" s="11">
+    <row r="14" ht="30" customHeight="1" s="12">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Step 2</t>
@@ -682,7 +682,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="30" customHeight="1" s="11">
+    <row r="15" ht="30" customHeight="1" s="12">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Step 3</t>
@@ -694,7 +694,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1" s="11">
+    <row r="16" ht="30" customHeight="1" s="12">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Step 4</t>
@@ -706,7 +706,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="30" customHeight="1" s="11">
+    <row r="17" ht="30" customHeight="1" s="12">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Step 5</t>
@@ -718,11 +718,11 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1" s="11">
+    <row r="18" ht="18" customHeight="1" s="12">
       <c r="A18" s="3" t="n"/>
       <c r="B18" s="2" t="n"/>
     </row>
-    <row r="19" ht="18" customHeight="1" s="11">
+    <row r="19" ht="18" customHeight="1" s="12">
       <c r="A19" s="1" t="inlineStr">
         <is>
           <t>RULES</t>
@@ -730,7 +730,7 @@
       </c>
       <c r="B19" s="2" t="n"/>
     </row>
-    <row r="20" ht="18" customHeight="1" s="11">
+    <row r="20" ht="18" customHeight="1" s="12">
       <c r="A20" s="3" t="inlineStr">
         <is>
           <t>Do not rename sheets</t>
@@ -742,7 +742,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="30" customHeight="1" s="11">
+    <row r="21" ht="30" customHeight="1" s="12">
       <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Do not rename column headers</t>
@@ -754,7 +754,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1" s="11">
+    <row r="22" ht="18" customHeight="1" s="12">
       <c r="A22" s="3" t="inlineStr">
         <is>
           <t>Keep the key column</t>
@@ -766,7 +766,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="30" customHeight="1" s="11">
+    <row r="23" ht="30" customHeight="1" s="12">
       <c r="A23" s="3" t="inlineStr">
         <is>
           <t>Mark status</t>
@@ -778,11 +778,11 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1" s="11">
+    <row r="24" ht="18" customHeight="1" s="12">
       <c r="A24" s="3" t="n"/>
       <c r="B24" s="2" t="n"/>
     </row>
-    <row r="25" ht="18" customHeight="1" s="11">
+    <row r="25" ht="18" customHeight="1" s="12">
       <c r="A25" s="3" t="inlineStr">
         <is>
           <t>Version</t>
@@ -794,7 +794,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="18" customHeight="1" s="11">
+    <row r="26" ht="18" customHeight="1" s="12">
       <c r="A26" s="3" t="inlineStr">
         <is>
           <t>Maintained by</t>
@@ -823,14 +823,14 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="8" customWidth="1" style="11" min="1" max="1"/>
-    <col width="18" customWidth="1" style="11" min="2" max="3"/>
-    <col width="12" customWidth="1" style="11" min="4" max="5"/>
-    <col width="10" customWidth="1" style="11" min="6" max="7"/>
-    <col width="45" customWidth="1" style="11" min="8" max="8"/>
+    <col width="8" customWidth="1" style="12" min="1" max="1"/>
+    <col width="18" customWidth="1" style="12" min="2" max="3"/>
+    <col width="12" customWidth="1" style="12" min="4" max="5"/>
+    <col width="10" customWidth="1" style="12" min="6" max="7"/>
+    <col width="45" customWidth="1" style="12" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" s="11">
+    <row r="1" ht="22" customHeight="1" s="12">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>code</t>
@@ -877,7 +877,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="36" customHeight="1" s="11">
+    <row r="2" ht="36" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>en</t>
@@ -924,7 +924,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" s="11">
+    <row r="3" ht="36" customHeight="1" s="12">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>de</t>
@@ -971,7 +971,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" s="11">
+    <row r="4" ht="36" customHeight="1" s="12">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>fr</t>
@@ -997,7 +997,7 @@
           <t>fr</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -1018,7 +1018,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" s="11">
+    <row r="5" ht="36" customHeight="1" s="12">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>nl</t>
@@ -1044,7 +1044,7 @@
           <t>nl</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" s="11">
+    <row r="6" ht="36" customHeight="1" s="12">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>zh</t>
@@ -1091,7 +1091,7 @@
           <t>zh-Hans</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F6" s="5" t="inlineStr">
         <is>
           <t>draft</t>
         </is>
@@ -1112,7 +1112,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" s="11">
+    <row r="7" ht="36" customHeight="1" s="12">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>vi</t>
@@ -1161,6 +1161,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -1173,16 +1174,16 @@
   <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="11" min="1" max="1"/>
-    <col width="25" customWidth="1" style="11" min="2" max="2"/>
-    <col width="40" customWidth="1" style="11" min="3" max="3"/>
-    <col width="20" customWidth="1" style="11" min="4" max="4"/>
-    <col width="40" customWidth="1" style="11" min="5" max="6"/>
-    <col width="25" customWidth="1" style="11" min="7" max="7"/>
-    <col width="35" customWidth="1" style="11" min="8" max="8"/>
+    <col width="10" customWidth="1" style="12" min="1" max="1"/>
+    <col width="25" customWidth="1" style="12" min="2" max="2"/>
+    <col width="40" customWidth="1" style="12" min="3" max="3"/>
+    <col width="20" customWidth="1" style="12" min="4" max="4"/>
+    <col width="40" customWidth="1" style="12" min="5" max="6"/>
+    <col width="25" customWidth="1" style="12" min="7" max="7"/>
+    <col width="35" customWidth="1" style="12" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" s="11">
+    <row r="1" ht="22" customHeight="1" s="12">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>language</t>
@@ -1224,7 +1225,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="72" customHeight="1" s="11">
+    <row r="2" ht="72" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>en</t>
@@ -1266,7 +1267,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="72" customHeight="1" s="11">
+    <row r="3" ht="72" customHeight="1" s="12">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>de</t>
@@ -1308,7 +1309,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="72" customHeight="1" s="11">
+    <row r="4" ht="72" customHeight="1" s="12">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>fr</t>
@@ -1350,7 +1351,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="72" customHeight="1" s="11">
+    <row r="5" ht="72" customHeight="1" s="12">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>nl</t>
@@ -1392,7 +1393,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="72" customHeight="1" s="11">
+    <row r="6" ht="72" customHeight="1" s="12">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>zh</t>
@@ -1434,7 +1435,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="72" customHeight="1" s="11">
+    <row r="7" ht="72" customHeight="1" s="12">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>vi</t>
@@ -1490,14 +1491,14 @@
   <dimension ref="A1:J144"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" style="11" min="1" max="1"/>
-    <col width="14" customWidth="1" style="11" min="2" max="2"/>
-    <col width="30" customWidth="1" style="11" min="3" max="3"/>
-    <col width="45" customWidth="1" style="11" min="4" max="6"/>
-    <col width="28" customWidth="1" style="11" min="7" max="8"/>
+    <col width="28" customWidth="1" style="12" min="1" max="1"/>
+    <col width="14" customWidth="1" style="12" min="2" max="2"/>
+    <col width="30" customWidth="1" style="12" min="3" max="3"/>
+    <col width="45" customWidth="1" style="12" min="4" max="6"/>
+    <col width="28" customWidth="1" style="12" min="7" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" s="11">
+    <row r="1" ht="22" customHeight="1" s="12">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>key</t>
@@ -1550,13 +1551,13 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  NAV</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="36" customHeight="1" s="11">
+    <row r="3" ht="36" customHeight="1" s="12">
       <c r="A3" s="7" t="inlineStr">
         <is>
           <t>nav.section_label</t>
@@ -1608,7 +1609,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="36" customHeight="1" s="11">
+    <row r="4" ht="36" customHeight="1" s="12">
       <c r="A4" s="7" t="inlineStr">
         <is>
           <t>nav.link.vision</t>
@@ -1660,7 +1661,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="36" customHeight="1" s="11">
+    <row r="5" ht="36" customHeight="1" s="12">
       <c r="A5" s="7" t="inlineStr">
         <is>
           <t>nav.link.gears</t>
@@ -1712,7 +1713,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="36" customHeight="1" s="11">
+    <row r="6" ht="36" customHeight="1" s="12">
       <c r="A6" s="7" t="inlineStr">
         <is>
           <t>nav.link.outputs</t>
@@ -1764,7 +1765,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="36" customHeight="1" s="11">
+    <row r="7" ht="36" customHeight="1" s="12">
       <c r="A7" s="7" t="inlineStr">
         <is>
           <t>nav.link.case</t>
@@ -1816,7 +1817,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="36" customHeight="1" s="11">
+    <row r="8" ht="36" customHeight="1" s="12">
       <c r="A8" s="7" t="inlineStr">
         <is>
           <t>nav.link.about</t>
@@ -1868,7 +1869,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="36" customHeight="1" s="11">
+    <row r="9" ht="36" customHeight="1" s="12">
       <c r="A9" s="7" t="inlineStr">
         <is>
           <t>nav.cta</t>
@@ -1921,13 +1922,13 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  HERO</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="36" customHeight="1" s="11">
+    <row r="11" ht="36" customHeight="1" s="12">
       <c r="A11" s="7" t="inlineStr">
         <is>
           <t>hero.eyebrow</t>
@@ -1979,7 +1980,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="36" customHeight="1" s="11">
+    <row r="12" ht="36" customHeight="1" s="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
           <t>hero.h1</t>
@@ -2031,7 +2032,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="36" customHeight="1" s="11">
+    <row r="13" ht="36" customHeight="1" s="12">
       <c r="A13" s="7" t="inlineStr">
         <is>
           <t>hero.sub</t>
@@ -2083,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="36" customHeight="1" s="11">
+    <row r="14" ht="36" customHeight="1" s="12">
       <c r="A14" s="7" t="inlineStr">
         <is>
           <t>hero.support</t>
@@ -2135,7 +2136,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="36" customHeight="1" s="11">
+    <row r="15" ht="36" customHeight="1" s="12">
       <c r="A15" s="7" t="inlineStr">
         <is>
           <t>hero.cta.primary</t>
@@ -2187,7 +2188,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="36" customHeight="1" s="11">
+    <row r="16" ht="36" customHeight="1" s="12">
       <c r="A16" s="7" t="inlineStr">
         <is>
           <t>hero.cta.secondary</t>
@@ -2240,13 +2241,13 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  STATS</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="36" customHeight="1" s="11">
+    <row r="18" ht="36" customHeight="1" s="12">
       <c r="A18" s="7" t="inlineStr">
         <is>
           <t>stat.1.label</t>
@@ -2298,7 +2299,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="36" customHeight="1" s="11">
+    <row r="19" ht="36" customHeight="1" s="12">
       <c r="A19" s="7" t="inlineStr">
         <is>
           <t>stat.2.label</t>
@@ -2350,7 +2351,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="36" customHeight="1" s="11">
+    <row r="20" ht="36" customHeight="1" s="12">
       <c r="A20" s="7" t="inlineStr">
         <is>
           <t>stat.3.label</t>
@@ -2402,7 +2403,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="36" customHeight="1" s="11">
+    <row r="21" ht="36" customHeight="1" s="12">
       <c r="A21" s="7" t="inlineStr">
         <is>
           <t>stat.4.label</t>
@@ -2454,7 +2455,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="36" customHeight="1" s="11">
+    <row r="22" ht="36" customHeight="1" s="12">
       <c r="A22" s="7" t="inlineStr">
         <is>
           <t>stat.tag</t>
@@ -2507,13 +2508,13 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  SHIFT</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="36" customHeight="1" s="11">
+    <row r="24" ht="36" customHeight="1" s="12">
       <c r="A24" s="7" t="inlineStr">
         <is>
           <t>shift.section_label</t>
@@ -2565,7 +2566,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="36" customHeight="1" s="11">
+    <row r="25" ht="36" customHeight="1" s="12">
       <c r="A25" s="7" t="inlineStr">
         <is>
           <t>shift.h</t>
@@ -2617,7 +2618,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="36" customHeight="1" s="11">
+    <row r="26" ht="36" customHeight="1" s="12">
       <c r="A26" s="7" t="inlineStr">
         <is>
           <t>shift.p1</t>
@@ -2669,7 +2670,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="36" customHeight="1" s="11">
+    <row r="27" ht="36" customHeight="1" s="12">
       <c r="A27" s="7" t="inlineStr">
         <is>
           <t>shift.p2</t>
@@ -2721,7 +2722,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="36" customHeight="1" s="11">
+    <row r="28" ht="36" customHeight="1" s="12">
       <c r="A28" s="7" t="inlineStr">
         <is>
           <t>shift.p3</t>
@@ -2773,7 +2774,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="36" customHeight="1" s="11">
+    <row r="29" ht="36" customHeight="1" s="12">
       <c r="A29" s="7" t="inlineStr">
         <is>
           <t>shift.quote</t>
@@ -2829,7 +2830,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="36" customHeight="1" s="11">
+    <row r="30" ht="36" customHeight="1" s="12">
       <c r="A30" t="inlineStr">
         <is>
           <t>shift.list.1</t>
@@ -2861,7 +2862,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="36" customHeight="1" s="11">
+    <row r="31" ht="36" customHeight="1" s="12">
       <c r="A31" t="inlineStr">
         <is>
           <t>shift.list.2</t>
@@ -2925,7 +2926,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="36" customHeight="1" s="11">
+    <row r="33" ht="36" customHeight="1" s="12">
       <c r="A33" t="inlineStr">
         <is>
           <t>shift.list.4</t>
@@ -2957,7 +2958,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="36" customHeight="1" s="11">
+    <row r="34" ht="36" customHeight="1" s="12">
       <c r="A34" t="inlineStr">
         <is>
           <t>shift.list.5</t>
@@ -2989,7 +2990,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="36" customHeight="1" s="11">
+    <row r="35" ht="36" customHeight="1" s="12">
       <c r="A35" s="7" t="inlineStr">
         <is>
           <t>struct.label</t>
@@ -3041,7 +3042,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="36" customHeight="1" s="11">
+    <row r="36" ht="36" customHeight="1" s="12">
       <c r="A36" s="7" t="inlineStr">
         <is>
           <t>struct.quote</t>
@@ -3094,13 +3095,13 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="A37" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  VISION</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="36" customHeight="1" s="11">
+    <row r="38" ht="36" customHeight="1" s="12">
       <c r="A38" s="7" t="inlineStr">
         <is>
           <t>vision.section_label</t>
@@ -3152,7 +3153,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="36" customHeight="1" s="11">
+    <row r="39" ht="36" customHeight="1" s="12">
       <c r="A39" s="7" t="inlineStr">
         <is>
           <t>vision.h</t>
@@ -3204,7 +3205,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="36" customHeight="1" s="11">
+    <row r="40" ht="36" customHeight="1" s="12">
       <c r="A40" s="7" t="inlineStr">
         <is>
           <t>vision.fear.intro</t>
@@ -3256,7 +3257,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="36" customHeight="1" s="11">
+    <row r="41" ht="36" customHeight="1" s="12">
       <c r="A41" s="7" t="inlineStr">
         <is>
           <t>vision.kl</t>
@@ -3312,14 +3313,14 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="36" customHeight="1" s="11">
-      <c r="A42" s="12" t="inlineStr">
+    <row r="42" ht="36" customHeight="1" s="12">
+      <c r="A42" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  GEARS</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="36" customHeight="1" s="11">
+    <row r="43" ht="36" customHeight="1" s="12">
       <c r="A43" s="7" t="inlineStr">
         <is>
           <t>gears.section_label</t>
@@ -3371,7 +3372,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="36" customHeight="1" s="11">
+    <row r="44" ht="36" customHeight="1" s="12">
       <c r="A44" s="7" t="inlineStr">
         <is>
           <t>gears.h</t>
@@ -3423,7 +3424,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="36" customHeight="1" s="11">
+    <row r="45" ht="36" customHeight="1" s="12">
       <c r="A45" s="7" t="inlineStr">
         <is>
           <t>gears.intro.p1</t>
@@ -3475,7 +3476,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="36" customHeight="1" s="11">
+    <row r="46" ht="36" customHeight="1" s="12">
       <c r="A46" s="7" t="inlineStr">
         <is>
           <t>gears.intro.p2</t>
@@ -3527,7 +3528,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="36" customHeight="1" s="11">
+    <row r="47" ht="36" customHeight="1" s="12">
       <c r="A47" s="7" t="inlineStr">
         <is>
           <t>gears.intro.p3</t>
@@ -3579,7 +3580,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="36" customHeight="1" s="11">
+    <row r="48" ht="36" customHeight="1" s="12">
       <c r="A48" s="7" t="inlineStr">
         <is>
           <t>gears.step1.title</t>
@@ -3638,7 +3639,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="36" customHeight="1" s="11">
+    <row r="50" ht="36" customHeight="1" s="12">
       <c r="A50" s="7" t="inlineStr">
         <is>
           <t>gears.step3.title</t>
@@ -3690,7 +3691,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="36" customHeight="1" s="11">
+    <row r="51" ht="36" customHeight="1" s="12">
       <c r="A51" s="7" t="inlineStr">
         <is>
           <t>gears.kl</t>
@@ -3742,7 +3743,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="36" customHeight="1" s="11">
+    <row r="52" ht="36" customHeight="1" s="12">
       <c r="A52" s="7" t="inlineStr">
         <is>
           <t>gears.naming.title</t>
@@ -3794,7 +3795,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="36" customHeight="1" s="11">
+    <row r="53" ht="36" customHeight="1" s="12">
       <c r="A53" s="7" t="inlineStr">
         <is>
           <t>gears.naming.body</t>
@@ -3846,14 +3847,14 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="36" customHeight="1" s="11">
-      <c r="A54" s="12" t="inlineStr">
+    <row r="54" ht="36" customHeight="1" s="12">
+      <c r="A54" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  OUTPUTS</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="36" customHeight="1" s="11">
+    <row r="55" ht="36" customHeight="1" s="12">
       <c r="A55" s="7" t="inlineStr">
         <is>
           <t>outputs.section_label</t>
@@ -3905,7 +3906,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="36" customHeight="1" s="11">
+    <row r="56" ht="36" customHeight="1" s="12">
       <c r="A56" s="7" t="inlineStr">
         <is>
           <t>outputs.h</t>
@@ -3961,7 +3962,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="36" customHeight="1" s="11">
+    <row r="57" ht="36" customHeight="1" s="12">
       <c r="A57" s="7" t="inlineStr">
         <is>
           <t>outputs.intro.p1</t>
@@ -4013,7 +4014,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="36" customHeight="1" s="11">
+    <row r="58" ht="36" customHeight="1" s="12">
       <c r="A58" s="7" t="inlineStr">
         <is>
           <t>outputs.intro.p2</t>
@@ -4065,7 +4066,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="36" customHeight="1" s="11">
+    <row r="59" ht="36" customHeight="1" s="12">
       <c r="A59" s="7" t="inlineStr">
         <is>
           <t>output.1.label</t>
@@ -4117,7 +4118,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="36" customHeight="1" s="11">
+    <row r="60" ht="36" customHeight="1" s="12">
       <c r="A60" s="7" t="inlineStr">
         <is>
           <t>output.1.title</t>
@@ -4169,7 +4170,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="36" customHeight="1" s="11">
+    <row r="61" ht="36" customHeight="1" s="12">
       <c r="A61" s="7" t="inlineStr">
         <is>
           <t>output.2.label</t>
@@ -4221,7 +4222,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="36" customHeight="1" s="11">
+    <row r="62" ht="36" customHeight="1" s="12">
       <c r="A62" s="7" t="inlineStr">
         <is>
           <t>output.2.title</t>
@@ -4305,7 +4306,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="36" customHeight="1" s="11">
+    <row r="64" ht="36" customHeight="1" s="12">
       <c r="A64" s="7" t="inlineStr">
         <is>
           <t>output.4.title</t>
@@ -4357,7 +4358,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="36" customHeight="1" s="11">
+    <row r="65" ht="36" customHeight="1" s="12">
       <c r="A65" s="7" t="inlineStr">
         <is>
           <t>output.5.title</t>
@@ -4409,7 +4410,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="36" customHeight="1" s="11">
+    <row r="66" ht="36" customHeight="1" s="12">
       <c r="A66" s="7" t="inlineStr">
         <is>
           <t>output.6.title</t>
@@ -4461,7 +4462,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="36" customHeight="1" s="11">
+    <row r="67" ht="36" customHeight="1" s="12">
       <c r="A67" s="7" t="inlineStr">
         <is>
           <t>outputs.foot</t>
@@ -4513,8 +4514,8 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="36" customHeight="1" s="11">
-      <c r="A68" s="12" t="inlineStr">
+    <row r="68" ht="36" customHeight="1" s="12">
+      <c r="A68" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  CASE</t>
         </is>
@@ -4527,7 +4528,7 @@
         </is>
       </c>
     </row>
-    <row r="70" ht="36" customHeight="1" s="11">
+    <row r="70" ht="36" customHeight="1" s="12">
       <c r="A70" s="7" t="inlineStr">
         <is>
           <t>case.tag</t>
@@ -4579,7 +4580,7 @@
         </is>
       </c>
     </row>
-    <row r="71" ht="36" customHeight="1" s="11">
+    <row r="71" ht="36" customHeight="1" s="12">
       <c r="A71" s="7" t="inlineStr">
         <is>
           <t>case.h</t>
@@ -4631,7 +4632,7 @@
         </is>
       </c>
     </row>
-    <row r="72" ht="36" customHeight="1" s="11">
+    <row r="72" ht="36" customHeight="1" s="12">
       <c r="A72" s="7" t="inlineStr">
         <is>
           <t>case.sub</t>
@@ -4683,7 +4684,7 @@
         </is>
       </c>
     </row>
-    <row r="73" ht="36" customHeight="1" s="11">
+    <row r="73" ht="36" customHeight="1" s="12">
       <c r="A73" s="7" t="inlineStr">
         <is>
           <t>case.kl</t>
@@ -4735,14 +4736,14 @@
         </is>
       </c>
     </row>
-    <row r="74" ht="36" customHeight="1" s="11">
-      <c r="A74" s="12" t="inlineStr">
+    <row r="74" ht="36" customHeight="1" s="12">
+      <c r="A74" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  FOR</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="36" customHeight="1" s="11">
+    <row r="75" ht="36" customHeight="1" s="12">
       <c r="A75" s="7" t="inlineStr">
         <is>
           <t>for.section_label</t>
@@ -4826,7 +4827,7 @@
         </is>
       </c>
     </row>
-    <row r="77" ht="36" customHeight="1" s="11">
+    <row r="77" ht="36" customHeight="1" s="12">
       <c r="A77" s="7" t="inlineStr">
         <is>
           <t>for.founders.role</t>
@@ -4878,7 +4879,7 @@
         </is>
       </c>
     </row>
-    <row r="78" ht="36" customHeight="1" s="11">
+    <row r="78" ht="36" customHeight="1" s="12">
       <c r="A78" s="7" t="inlineStr">
         <is>
           <t>for.founders.body</t>
@@ -4930,7 +4931,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="36" customHeight="1" s="11">
+    <row r="79" ht="36" customHeight="1" s="12">
       <c r="A79" s="7" t="inlineStr">
         <is>
           <t>for.operators.role</t>
@@ -4982,7 +4983,7 @@
         </is>
       </c>
     </row>
-    <row r="80" ht="36" customHeight="1" s="11">
+    <row r="80" ht="36" customHeight="1" s="12">
       <c r="A80" s="7" t="inlineStr">
         <is>
           <t>for.investors.role</t>
@@ -5034,14 +5035,14 @@
         </is>
       </c>
     </row>
-    <row r="81" ht="36" customHeight="1" s="11">
-      <c r="A81" s="12" t="inlineStr">
+    <row r="81" ht="36" customHeight="1" s="12">
+      <c r="A81" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  LADDER</t>
         </is>
       </c>
     </row>
-    <row r="82" ht="36" customHeight="1" s="11">
+    <row r="82" ht="36" customHeight="1" s="12">
       <c r="A82" s="7" t="inlineStr">
         <is>
           <t>ladder.section_label</t>
@@ -5093,7 +5094,7 @@
         </is>
       </c>
     </row>
-    <row r="83" ht="36" customHeight="1" s="11">
+    <row r="83" ht="36" customHeight="1" s="12">
       <c r="A83" s="7" t="inlineStr">
         <is>
           <t>ladder.h</t>
@@ -5149,7 +5150,7 @@
         </is>
       </c>
     </row>
-    <row r="84" ht="36" customHeight="1" s="11">
+    <row r="84" ht="36" customHeight="1" s="12">
       <c r="A84" s="7" t="inlineStr">
         <is>
           <t>ladder.sub</t>
@@ -5233,7 +5234,7 @@
         </is>
       </c>
     </row>
-    <row r="86" ht="36" customHeight="1" s="11">
+    <row r="86" ht="36" customHeight="1" s="12">
       <c r="A86" s="7" t="inlineStr">
         <is>
           <t>ladder.step2.title</t>
@@ -5285,7 +5286,7 @@
         </is>
       </c>
     </row>
-    <row r="87" ht="36" customHeight="1" s="11">
+    <row r="87" ht="36" customHeight="1" s="12">
       <c r="A87" s="7" t="inlineStr">
         <is>
           <t>ladder.step3.title</t>
@@ -5337,7 +5338,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="36" customHeight="1" s="11">
+    <row r="88" ht="36" customHeight="1" s="12">
       <c r="A88" s="7" t="inlineStr">
         <is>
           <t>ladder.step4.title</t>
@@ -5421,14 +5422,14 @@
         </is>
       </c>
     </row>
-    <row r="90" ht="36" customHeight="1" s="11">
-      <c r="A90" s="12" t="inlineStr">
+    <row r="90" ht="36" customHeight="1" s="12">
+      <c r="A90" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  TESTI</t>
         </is>
       </c>
     </row>
-    <row r="91" ht="36" customHeight="1" s="11">
+    <row r="91" ht="36" customHeight="1" s="12">
       <c r="A91" s="7" t="inlineStr">
         <is>
           <t>testi.section_label</t>
@@ -5480,7 +5481,7 @@
         </is>
       </c>
     </row>
-    <row r="92" ht="36" customHeight="1" s="11">
+    <row r="92" ht="36" customHeight="1" s="12">
       <c r="A92" s="7" t="inlineStr">
         <is>
           <t>testi.quote</t>
@@ -5532,7 +5533,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="36" customHeight="1" s="11">
+    <row r="93" ht="36" customHeight="1" s="12">
       <c r="A93" s="7" t="inlineStr">
         <is>
           <t>testi.attr</t>
@@ -5584,8 +5585,8 @@
         </is>
       </c>
     </row>
-    <row r="94" ht="36" customHeight="1" s="11">
-      <c r="A94" s="12" t="inlineStr">
+    <row r="94" ht="36" customHeight="1" s="12">
+      <c r="A94" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  ABOUT</t>
         </is>
@@ -5598,7 +5599,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="36" customHeight="1" s="11">
+    <row r="96" ht="36" customHeight="1" s="12">
       <c r="A96" s="7" t="inlineStr">
         <is>
           <t>about.h</t>
@@ -5650,7 +5651,7 @@
         </is>
       </c>
     </row>
-    <row r="97" ht="36" customHeight="1" s="11">
+    <row r="97" ht="36" customHeight="1" s="12">
       <c r="A97" s="7" t="inlineStr">
         <is>
           <t>about.letter.salutation</t>
@@ -5702,7 +5703,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="36" customHeight="1" s="11">
+    <row r="98" ht="36" customHeight="1" s="12">
       <c r="A98" s="7" t="inlineStr">
         <is>
           <t>about.sig</t>
@@ -5754,7 +5755,7 @@
         </is>
       </c>
     </row>
-    <row r="99" ht="36" customHeight="1" s="11">
+    <row r="99" ht="36" customHeight="1" s="12">
       <c r="A99" s="7" t="inlineStr">
         <is>
           <t>about.belief.title</t>
@@ -5806,14 +5807,14 @@
         </is>
       </c>
     </row>
-    <row r="100" ht="36" customHeight="1" s="11">
-      <c r="A100" s="12" t="inlineStr">
+    <row r="100" ht="36" customHeight="1" s="12">
+      <c r="A100" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  START</t>
         </is>
       </c>
     </row>
-    <row r="101" ht="36" customHeight="1" s="11">
+    <row r="101" ht="36" customHeight="1" s="12">
       <c r="A101" s="7" t="inlineStr">
         <is>
           <t>start.section_label</t>
@@ -5865,7 +5866,7 @@
         </is>
       </c>
     </row>
-    <row r="102" ht="36" customHeight="1" s="11">
+    <row r="102" ht="36" customHeight="1" s="12">
       <c r="A102" s="7" t="inlineStr">
         <is>
           <t>start.h</t>
@@ -5917,7 +5918,7 @@
         </is>
       </c>
     </row>
-    <row r="103" ht="36" customHeight="1" s="11">
+    <row r="103" ht="36" customHeight="1" s="12">
       <c r="A103" s="7" t="inlineStr">
         <is>
           <t>start.sub</t>
@@ -5969,7 +5970,7 @@
         </is>
       </c>
     </row>
-    <row r="104" ht="36" customHeight="1" s="11">
+    <row r="104" ht="36" customHeight="1" s="12">
       <c r="A104" s="7" t="inlineStr">
         <is>
           <t>start.kl</t>
@@ -6021,7 +6022,7 @@
         </is>
       </c>
     </row>
-    <row r="105" ht="36" customHeight="1" s="11">
+    <row r="105" ht="36" customHeight="1" s="12">
       <c r="A105" s="7" t="inlineStr">
         <is>
           <t>form.intro</t>
@@ -6073,7 +6074,7 @@
         </is>
       </c>
     </row>
-    <row r="106" ht="36" customHeight="1" s="11">
+    <row r="106" ht="36" customHeight="1" s="12">
       <c r="A106" s="7" t="inlineStr">
         <is>
           <t>form.label.name</t>
@@ -6157,7 +6158,7 @@
         </is>
       </c>
     </row>
-    <row r="108" ht="36" customHeight="1" s="11">
+    <row r="108" ht="36" customHeight="1" s="12">
       <c r="A108" s="7" t="inlineStr">
         <is>
           <t>form.label.email</t>
@@ -6209,7 +6210,7 @@
         </is>
       </c>
     </row>
-    <row r="109" ht="36" customHeight="1" s="11">
+    <row r="109" ht="36" customHeight="1" s="12">
       <c r="A109" s="7" t="inlineStr">
         <is>
           <t>form.label.message</t>
@@ -6261,7 +6262,7 @@
         </is>
       </c>
     </row>
-    <row r="110" ht="36" customHeight="1" s="11">
+    <row r="110" ht="36" customHeight="1" s="12">
       <c r="A110" s="7" t="inlineStr">
         <is>
           <t>form.placeholder.message</t>
@@ -6313,7 +6314,7 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="36" customHeight="1" s="11">
+    <row r="111" ht="36" customHeight="1" s="12">
       <c r="A111" s="7" t="inlineStr">
         <is>
           <t>form.btn</t>
@@ -6366,13 +6367,13 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="12" t="inlineStr">
+      <c r="A112" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  CTA</t>
         </is>
       </c>
     </row>
-    <row r="113" ht="36" customHeight="1" s="11">
+    <row r="113" ht="36" customHeight="1" s="12">
       <c r="A113" s="7" t="inlineStr">
         <is>
           <t>cta.h</t>
@@ -6424,7 +6425,7 @@
         </is>
       </c>
     </row>
-    <row r="114" ht="36" customHeight="1" s="11">
+    <row r="114" ht="36" customHeight="1" s="12">
       <c r="A114" s="7" t="inlineStr">
         <is>
           <t>cta.body</t>
@@ -6476,7 +6477,7 @@
         </is>
       </c>
     </row>
-    <row r="115" ht="36" customHeight="1" s="11">
+    <row r="115" ht="36" customHeight="1" s="12">
       <c r="A115" s="7" t="inlineStr">
         <is>
           <t>cta.btn.primary</t>
@@ -6528,7 +6529,7 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="36" customHeight="1" s="11">
+    <row r="116" ht="36" customHeight="1" s="12">
       <c r="A116" s="7" t="inlineStr">
         <is>
           <t>cta.btn.secondary</t>
@@ -6580,8 +6581,8 @@
         </is>
       </c>
     </row>
-    <row r="117" ht="36" customHeight="1" s="11">
-      <c r="A117" s="12" t="inlineStr">
+    <row r="117" ht="36" customHeight="1" s="12">
+      <c r="A117" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  FOOTER</t>
         </is>
@@ -6619,7 +6620,7 @@
         </is>
       </c>
     </row>
-    <row r="119" ht="36" customHeight="1" s="11">
+    <row r="119" ht="36" customHeight="1" s="12">
       <c r="A119" s="7" t="inlineStr">
         <is>
           <t>footer.col.explore</t>
@@ -6671,7 +6672,7 @@
         </is>
       </c>
     </row>
-    <row r="120" ht="36" customHeight="1" s="11">
+    <row r="120" ht="36" customHeight="1" s="12">
       <c r="A120" s="7" t="inlineStr">
         <is>
           <t>footer.col.contact</t>
@@ -6723,7 +6724,7 @@
         </is>
       </c>
     </row>
-    <row r="121">
+    <row r="121" ht="26" customHeight="1" s="12">
       <c r="A121" s="7" t="inlineStr">
         <is>
           <t>footer.copyright</t>
@@ -6775,7 +6776,7 @@
         </is>
       </c>
     </row>
-    <row r="122">
+    <row r="122" ht="65" customHeight="1" s="12">
       <c r="A122" s="7" t="inlineStr">
         <is>
           <t>footer.descriptor</t>
@@ -6828,13 +6829,13 @@
       </c>
     </row>
     <row r="123">
-      <c r="A123" s="12" t="inlineStr">
+      <c r="A123" s="10" t="inlineStr">
         <is>
           <t xml:space="preserve">  META</t>
         </is>
       </c>
     </row>
-    <row r="124">
+    <row r="124" ht="78" customHeight="1" s="12">
       <c r="A124" s="7" t="inlineStr">
         <is>
           <t>page.title</t>
@@ -7638,12 +7639,12 @@
   <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="11" min="1" max="1"/>
-    <col width="50" customWidth="1" style="11" min="2" max="2"/>
-    <col width="80" customWidth="1" style="11" min="3" max="3"/>
-    <col width="50" customWidth="1" style="11" min="4" max="4"/>
-    <col width="80" customWidth="1" style="11" min="5" max="5"/>
-    <col width="40" customWidth="1" style="11" min="6" max="6"/>
+    <col width="10" customWidth="1" style="12" min="1" max="1"/>
+    <col width="50" customWidth="1" style="12" min="2" max="2"/>
+    <col width="80" customWidth="1" style="12" min="3" max="3"/>
+    <col width="50" customWidth="1" style="12" min="4" max="4"/>
+    <col width="80" customWidth="1" style="12" min="5" max="5"/>
+    <col width="40" customWidth="1" style="12" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -7678,7 +7679,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="54" customHeight="1" s="11">
+    <row r="2" ht="54" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>en</t>
@@ -7710,7 +7711,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="54" customHeight="1" s="11">
+    <row r="3" ht="54" customHeight="1" s="12">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>de</t>
@@ -7742,7 +7743,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="54" customHeight="1" s="11">
+    <row r="4" ht="54" customHeight="1" s="12">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>fr</t>
@@ -7774,7 +7775,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="54" customHeight="1" s="11">
+    <row r="5" ht="54" customHeight="1" s="12">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>nl</t>
@@ -7806,7 +7807,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="54" customHeight="1" s="11">
+    <row r="6" ht="54" customHeight="1" s="12">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>zh</t>
@@ -7838,7 +7839,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="54" customHeight="1" s="11">
+    <row r="7" ht="54" customHeight="1" s="12">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>vi</t>
@@ -7884,15 +7885,15 @@
   <dimension ref="A1:I7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" style="11" min="1" max="1"/>
-    <col width="12" customWidth="1" style="11" min="2" max="2"/>
-    <col width="30" customWidth="1" style="11" min="3" max="4"/>
-    <col width="45" customWidth="1" style="11" min="5" max="5"/>
-    <col width="14" customWidth="1" style="11" min="6" max="7"/>
-    <col width="12" customWidth="1" style="11" min="8" max="9"/>
+    <col width="10" customWidth="1" style="12" min="1" max="1"/>
+    <col width="12" customWidth="1" style="12" min="2" max="2"/>
+    <col width="30" customWidth="1" style="12" min="3" max="4"/>
+    <col width="45" customWidth="1" style="12" min="5" max="5"/>
+    <col width="14" customWidth="1" style="12" min="6" max="7"/>
+    <col width="12" customWidth="1" style="12" min="8" max="9"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1" s="11">
+    <row r="1" ht="28" customHeight="1" s="12">
       <c r="A1" s="4" t="inlineStr">
         <is>
           <t>language</t>
@@ -7939,7 +7940,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="28" customHeight="1" s="11">
+    <row r="2" ht="28" customHeight="1" s="12">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t>en</t>
@@ -7986,7 +7987,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28" customHeight="1" s="11">
+    <row r="3" ht="28" customHeight="1" s="12">
       <c r="A3" s="2" t="inlineStr">
         <is>
           <t>de</t>
@@ -8033,7 +8034,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28" customHeight="1" s="11">
+    <row r="4" ht="28" customHeight="1" s="12">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>fr</t>
@@ -8080,7 +8081,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28" customHeight="1" s="11">
+    <row r="5" ht="28" customHeight="1" s="12">
       <c r="A5" s="2" t="inlineStr">
         <is>
           <t>nl</t>
@@ -8127,7 +8128,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="28" customHeight="1" s="11">
+    <row r="6" ht="28" customHeight="1" s="12">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>zh</t>
@@ -8174,7 +8175,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28" customHeight="1" s="11">
+    <row r="7" ht="28" customHeight="1" s="12">
       <c r="A7" s="2" t="inlineStr">
         <is>
           <t>vi</t>

</xml_diff>

<commit_message>
feat: launch French, Dutch and Chinese with full translations
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -997,9 +997,9 @@
           <t>fr</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>live</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1044,9 +1044,9 @@
           <t>nl</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>live</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1091,9 +1091,9 @@
           <t>zh-Hans</t>
         </is>
       </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>draft</t>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>live</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1741,7 +1741,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Livrables</t>
+          <t>Résultats</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1751,7 +1751,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>成果</t>
+          <t>交付成果</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Case Study</t>
+          <t>Casestudy</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -1855,7 +1855,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>关于</t>
+          <t>关于我们</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1897,17 +1897,17 @@
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Discutons</t>
+          <t>Parlez à GKIM</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Contact opnemen</t>
+          <t>Neem contact op met GKIM</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>联系我们</t>
+          <t>联系 GKIM</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1951,22 +1951,22 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
+          <t>Business-System-Design</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Conception de systèmes métier</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
           <t>Business System Design</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Conception de systèmes</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Systeem Ontwerp</t>
-        </is>
-      </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>商业系统设计</t>
+          <t>业务系统设计</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -2003,22 +2003,22 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Gestalten Sie Ihr KI-natives Geschäft</t>
+          <t>Gestalten Sie Ihr KI-natives Unternehmen</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Concevez votre entreprise native IA</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Ontwerp uw AI-native bedrijf</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>设计您的AI原生企业</t>
+          <t>设计您的 AI 原生业务</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -2055,22 +2055,22 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Wettbewerbsvorteil ist nicht länger strategisch. Er ist strukturell.</t>
+          <t>Wettbewerbsvorteil ist nicht mehr strategisch. Er ist strukturell.</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>L'avantage compétitif n'est plus stratégique. Il est structurel.</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Competitief voordeel is niet langer strategisch. Het is structureel.</t>
         </is>
       </c>
       <c r="H13" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>竞争优势不再是战略问题，而是结构问题。</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
@@ -2107,22 +2107,22 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Wir definieren die fehlende Schicht zwischen Strategie und Technik — wie Ihr Geschäft tatsächlich als System funktioniert, das Wert schafft.</t>
+          <t>Wir definieren die fehlende Ebene zwischen Strategie und Entwicklung — wie Ihr Unternehmen als System tatsächlich funktioniert, um Wert zu schaffen.</t>
         </is>
       </c>
       <c r="F14" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Nous définissons la couche manquante entre la stratégie et l'ingénierie — comment votre entreprise fonctionne réellement en tant que système conçu pour créer de la valeur.</t>
         </is>
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>We definiëren de ontbrekende laag tussen strategie en engineering — hoe uw bedrijf daadwerkelijk als een systeem werkt dat waarde creëert.</t>
         </is>
       </c>
       <c r="H14" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>我们定义了战略与工程之间缺失的层次——您的业务如何作为一个系统运作，以创造价值。</t>
         </is>
       </c>
       <c r="I14" s="6" t="inlineStr">
@@ -2164,17 +2164,17 @@
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Discutons</t>
+          <t>Parlez à GKIM</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Contact opnemen</t>
+          <t>Neem contact op met GKIM</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>联系我们</t>
+          <t>联系 GKIM</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -2216,17 +2216,17 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Voir les livrables</t>
+          <t>Découvrez ce que vous obtenez</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Bekijk resultaten</t>
+          <t>Zie wat u krijgt</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>查看成果</t>
+          <t>了解您将获得什么</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -2270,22 +2270,22 @@
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Entworfene Business Systeme</t>
+          <t>Entworfene Business-Systeme</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Systèmes métier conçus</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Business Systems Ontworpen</t>
         </is>
       </c>
       <c r="H18" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>已设计的业务系统</t>
         </is>
       </c>
       <c r="I18" s="6" t="inlineStr">
@@ -2322,22 +2322,22 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Strukturierte tägliche Transaktionen</t>
+          <t>Täglich strukturierte Transaktionen</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Transactions quotidiennes structurées</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Dagelijkse Transacties Gestructureerd</t>
         </is>
       </c>
       <c r="H19" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>已结构化的日交易量</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
@@ -2374,22 +2374,22 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Bereitgestellte Systeme</t>
+          <t>Gelieferte Systeme</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Systèmes livrés</t>
         </is>
       </c>
       <c r="G20" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Systemen Opgeleverd</t>
         </is>
       </c>
       <c r="H20" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>已交付的系统</t>
         </is>
       </c>
       <c r="I20" s="6" t="inlineStr">
@@ -2426,22 +2426,22 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Schnittstelle zwischen Strategie und Technik</t>
+          <t>Strategie- und Engineering-Schnittstelle</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Intersection stratégie et ingénierie</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Strategie &amp; Engineering Kruispunt</t>
         </is>
       </c>
       <c r="H21" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>战略与工程的交汇点</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
@@ -2478,22 +2478,22 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Von Tag eins für Skalierbarkeit ausgelegt — nicht später umgestaltet.</t>
+          <t>Von Tag eins für Skalierung ausgelegt — nicht später umgestaltet.</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Conçu pour l'échelle dès le premier jour — non refactorisé ultérieurement.</t>
         </is>
       </c>
       <c r="G22" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Ontworpen voor schaal vanaf dag één — niet later ervan afgeleid.</t>
         </is>
       </c>
       <c r="H22" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>从第一天起就为规模化设计——而非事后重构。</t>
         </is>
       </c>
       <c r="I22" s="6" t="inlineStr">
@@ -2542,7 +2542,7 @@
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Le Changement</t>
+          <t>Le changement</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2589,22 +2589,22 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Unternehmen beginnen anders auszusehen</t>
+          <t>Unternehmen beginnen, anders auszusehen</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Les entreprises commencent à avoir un autre aspect</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Bedrijven Zien Er Steeds Anders Uit</t>
         </is>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>业务正在呈现不同的样貌</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
@@ -2646,17 +2646,17 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>L'IA a donné à chaque entreprise la même vitesse de construction.</t>
         </is>
       </c>
       <c r="G26" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>AI heeft elk bedrijf dezelfde bouwsnelheid gegeven.</t>
         </is>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>AI 为每家公司提供了相同的构建速度。</t>
         </is>
       </c>
       <c r="I26" s="6" t="inlineStr">
@@ -2693,22 +2693,22 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Aber Geschwindigkeit spielt keine Rolle, wenn das Geschäft nie richtig als System definiert wurde. Dort scheitern die meisten digitalen Unternehmen.</t>
+          <t>Aber Geschwindigkeit ist nutzlos, wenn das Unternehmen nie als System richtig definiert wurde. Hier brechen die meisten digitalen Unternehmen zusammen.</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Mais la vitesse n'a pas d'importance si l'entreprise n'a jamais été correctement définie en tant que système. C'est là que la plupart des entreprises numériques échouent.</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Maar snelheid maakt niet uit als het bedrijf nooit goed als systeem is gedefinieerd. Dat is waar de meeste digitale bedrijven falen.</t>
         </is>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>但如果业务从未被恰当地定义为一个系统，速度就无关紧要。这正是大多数数字业务崩溃的地方。</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
@@ -2745,22 +2745,22 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>Die Einschränkung hat sich von der Entwicklung zur Definition verschoben.</t>
+          <t>Das Engpass hat sich von der Entwicklung zur Definition verschoben.</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>La contrainte s'est déplacée du développement à la définition.</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>De beperking is verschoven van ontwikkeling — naar definitie.</t>
         </is>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>制约因素已从开发转变为定义。</t>
         </is>
       </c>
       <c r="I28" s="6" t="inlineStr">
@@ -2804,17 +2804,20 @@
       </c>
       <c r="F29" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>La vitesse n'est pas l'avantage.
+La conception l'est.</t>
         </is>
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Snelheid is niet het voordeel.
+Ontwerp is.</t>
         </is>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>速度不是优势。
+设计才是。</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
@@ -2848,7 +2851,22 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Die meisten Unternehmen entdecken Probleme erst nach der Entwicklung</t>
+          <t>Die meisten Unternehmen entdecken Probleme erst nach dem Bau</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>La plupart des entreprises découvrent ce qui ne va pas après avoir construit</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>De meeste bedrijven ontdekken wat er mis is nadat zij het hebben gebouwd</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>大多数公司在构建后才发现问题所在</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -2883,6 +2901,21 @@
           <t>Anforderungen sind unvollständig, bevor die erste Codezeile geschrieben wird</t>
         </is>
       </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Les exigences sont incomplètes avant la première ligne de code</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Vereisten zijn onvolledig voordat de eerste regel code wordt geschreven</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>在编写第一行代码前，需求就不完整</t>
+        </is>
+      </c>
       <c r="I31" t="inlineStr">
         <is>
           <t>Các yêu cầu không hoàn chỉnh trước khi viết dòng mã đầu tiên</t>
@@ -2915,6 +2948,21 @@
           <t>Die Logik ist über Teams und Systeme hinweg inkonsistent</t>
         </is>
       </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>La logique est incohérente entre les équipes et les systèmes</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Logica is inconsistent tussen teams en systemen</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>逻辑在团队和系统间不一致</t>
+        </is>
+      </c>
       <c r="I32" t="inlineStr">
         <is>
           <t>Logic không nhất quán trên các team và hệ thống</t>
@@ -2944,7 +2992,22 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Stakeholder bleiben misaligned, bis die Umsetzung dies aufdeckt</t>
+          <t>Stakeholder bleiben uneinig, bis die Umsetzung es offenbart</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Les parties prenantes restent désalignées jusqu'à ce que l'exécution l'expose</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Stakeholders blijven niet aligned totdat uitvoering dit blootlegt</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>直到执行暴露问题，利益相关者才保持一致</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -2976,7 +3039,22 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Validierung erfolgt durch Entwicklung statt vorher</t>
+          <t>Validierung erfolgt durch Bau statt davor</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>La validation se fait par la construction plutôt qu'avant</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Validatie vindt plaats door te bouwen in plaats van daarvoor</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>验证是通过构建而非在构建前进行</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -3018,17 +3096,17 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Le principe fondamental de GEARS™</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Het kernprincipe van GEARS™</t>
         </is>
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ 的核心原则</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -3070,17 +3148,17 @@
       </c>
       <c r="F36" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>L'IA implémente la structure, non l'intention. Les modèles commerciaux doivent être exprimés comme des hiérarchies explicites.</t>
         </is>
       </c>
       <c r="G36" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>AI implementeert structuur, niet intentie. Businessmodellen moeten worden uitgedrukt als expliciete hiërarchieën.</t>
         </is>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>AI 实现结构，而非意图。业务模式必须表达为明确的层级。</t>
         </is>
       </c>
       <c r="I36" s="6" t="inlineStr">
@@ -3181,17 +3259,17 @@
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>L'entreprise native IA</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Het AI-native Bedrijf</t>
         </is>
       </c>
       <c r="H39" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>AI 原生业务</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -3228,22 +3306,22 @@
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>KI wirft berechtigte Fragen auf. Was passiert mit den Menschen in diesen Unternehmen? Was erleben Kunden? Was bedeutet es für Investoren? Die Antwort hängt vollständig davon ab, wie das System gestaltet ist.</t>
+          <t>KI wirft berechtigte Fragen auf. Was passiert mit den Menschen in diesen Unternehmen? Was erleben Kunden? Was bedeutet es für Investoren? Die Antwort hängt ganz davon ab, wie das System gestaltet ist.</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>L'IA soulève des questions légitimes. Qu'advient-il des personnes au sein de ces entreprises ? Qu'expérimentent les clients ? Qu'est-ce que cela signifie pour ceux qui investissent ? La réponse dépend entièrement de la conception du système.</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>AI roept rechtmatige vragen op. Wat gebeurt er met de mensen in deze bedrijven? Wat ervaren klanten? Wat betekent het voor degenen die investeren? Het antwoord hangt volledig af van hoe het systeem is ontworpen.</t>
         </is>
       </c>
       <c r="H40" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>AI 提出了合理的问题。这些业务内部的人会发生什么？客户会体验到什么？这对投资者意味着什么？答案完全取决于系统的设计方式。</t>
         </is>
       </c>
       <c r="I40" s="6" t="inlineStr">
@@ -3282,22 +3360,25 @@
       <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Nicht bessere Software.
-Ein besser gestaltetes Geschäft.</t>
+Ein bessser gestaltetes Unternehmen.</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Pas un meilleur logiciel.
+Une entreprise mieux conçue.</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Niet betere software.
+Een beter ontworpen bedrijf.</t>
         </is>
       </c>
       <c r="H41" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>不是更好的软件。
+而是设计更好的业务。</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -3343,22 +3424,22 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>GEARS™ — Business-gesteuertes System Design</t>
+          <t>GEARS™ — Business-gesteuertes System-Design</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ — Conception de systèmes dirigée par l'entreprise</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ — Business-Led System Design</t>
         </is>
       </c>
       <c r="H43" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ — 业务驱动的系统设计</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -3395,22 +3476,22 @@
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Definieren Sie das System, bevor Sie es aufbauen</t>
+          <t>Definieren Sie das System, bevor Sie es bauen</t>
         </is>
       </c>
       <c r="F44" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Définissez le système avant de le construire</t>
         </is>
       </c>
       <c r="G44" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Definieer het Systeem Voordat U Het Bouwt</t>
         </is>
       </c>
       <c r="H44" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>在构建前定义系统</t>
         </is>
       </c>
       <c r="I44" s="6" t="inlineStr">
@@ -3447,22 +3528,22 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>GEARS™ ist die Methode, die GKIM verwendet, um Geschäftsideen in funktionierende Geschäftsmaschinen umzuwandeln.</t>
+          <t>GEARS™ ist die Methode, die GKIM verwendet, um Geschäftsideen in funktionierende Business-Engines umzuwandeln.</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ est la méthode que GKIM utilise pour transformer les idées commerciales en moteurs commerciaux fonctionnels.</t>
         </is>
       </c>
       <c r="G45" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ is de methode die GKIM gebruikt om bedrijfsideeën in functionerende bedrijfsmotoren om te zetten.</t>
         </is>
       </c>
       <c r="H45" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ 是 GKIM 用来将业务创意转化为运行的业务引擎的方法。</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
@@ -3499,22 +3580,22 @@
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Sie beginnt nicht mit Features. Sie beginnt damit: wie das Geschäft tatsächlich arbeiten muss, um Wert zu schaffen.</t>
+          <t>Es beginnt nicht mit Features. Es beginnt mit: Wie das Unternehmen tatsächlich funktionieren muss, um Wert zu schaffen.</t>
         </is>
       </c>
       <c r="F46" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Elle ne commence pas par les fonctionnalités. Elle commence par : comment l'entreprise doit réellement fonctionner pour créer de la valeur.</t>
         </is>
       </c>
       <c r="G46" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Het begint niet met features. Het begint met: hoe het bedrijf daadwerkelijk moet werken om waarde te creëren.</t>
         </is>
       </c>
       <c r="H46" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>它不从功能开始，而是从以下问题开始：业务必须如何实际运作以创造价值。</t>
         </is>
       </c>
       <c r="I46" s="6" t="inlineStr">
@@ -3551,22 +3632,22 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Jedes Zahnrad ist eine benannte Einheit der Wertschöpfung — definiert durch das, was es produziert, nicht wie es arbeitet.</t>
+          <t>Jedes Zahnrad ist eine benannte Einheit der Wertschöpfung — definiert durch das, was es produziert, nicht wie es funktioniert.</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Chaque engrenage est une unité nommée de création de valeur — définie par ce qu'elle produit, non par son fonctionnement.</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Elk tandwiel is een benoemde eenheid van waardecreatie — gedefinieerd door wat het produceert, niet hoe het werkt.</t>
         </is>
       </c>
       <c r="H47" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>每个齿轮是一个具名的价值创造单元——由它产生什么来定义，而非如何操作。</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
@@ -3603,22 +3684,22 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Erkunden — Definieren Sie die Geschäftsmaschine</t>
+          <t>Entdecken — Definieren Sie die Business-Engine</t>
         </is>
       </c>
       <c r="F48" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Découvrir — Définir le moteur commercial</t>
         </is>
       </c>
       <c r="G48" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Ontdekken — Definieer de Bedrijfsmotor</t>
         </is>
       </c>
       <c r="H48" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>发现——定义业务引擎</t>
         </is>
       </c>
       <c r="I48" s="6" t="inlineStr">
@@ -3662,22 +3743,22 @@
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Liefern — Baureife Outputs</t>
+          <t>Liefern — Build-ready Outputs</t>
         </is>
       </c>
       <c r="F50" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Livrer — Résultats prêts à la construction</t>
         </is>
       </c>
       <c r="G50" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Opleveren — Build-Ready Resultaten</t>
         </is>
       </c>
       <c r="H50" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>交付——可构建的成果</t>
         </is>
       </c>
       <c r="I50" s="6" t="inlineStr">
@@ -3719,17 +3800,17 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ ne s'arrête pas à l'insight. Il produit la structure requise pour construire.</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ stopt niet bij inzicht. Het produceert de structuur die nodig is om te bouwen.</t>
         </is>
       </c>
       <c r="H51" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ 不仅仅提供洞见，它还提供构建所需的结构。</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -3766,22 +3847,22 @@
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Jedes Zahnrad wird mit einem Verb und einem Substantiv benannt. Präzise.</t>
+          <t>Jedes Zahnrad ist mit einem Verb und einem Nomen benannt. Präzise.</t>
         </is>
       </c>
       <c r="F52" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Chaque engrenage est nommé avec un verbe et un nom. Précisément.</t>
         </is>
       </c>
       <c r="G52" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Elk tandwiel wordt benoemd met een werkwoord en een zelfstandig naamwoord. Precies.</t>
         </is>
       </c>
       <c r="H52" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>每个齿轮都用动词和名词精确命名。</t>
         </is>
       </c>
       <c r="I52" s="6" t="inlineStr">
@@ -3818,22 +3899,22 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Ein Zahnradname ist ein Vertrag. Er erklärt, was das Zahnrad tut und worauf es einwirkt. Vage Namen verbergen Komplexität. Präzise Namen machen das System lesbar — und daher baubar.</t>
+          <t>Ein Zahnradname ist ein Vertrag. Er erklärt, was das Zahnrad tut und worum es sich kümmert. Vage Namen verbergen Komplexität. Präzise Namen machen das System verständlich — und daher baubar.</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Un nom d'engrenage est un contrat. Il déclare ce que l'engrenage fait et sur quoi il agit. Les noms vagues cachent la complexité. Les noms précis rendent le système lisible — et donc constructible.</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Een tandwielnaam is een contract. Het verklaart wat het tandwiel doet en waarop het inwerkt. Vage namen verbergen complexiteit. Nauwkeurige namen maken het systeem leesbaar — en dus bouwbaar.</t>
         </is>
       </c>
       <c r="H53" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>齿轮名称是一份契约。它声明齿轮做什么以及作用于什么。模糊的名称隐藏复杂性，精确的名称使系统清晰易懂——因此也可构建。</t>
         </is>
       </c>
       <c r="I53" s="6" t="inlineStr">
@@ -3877,22 +3958,22 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Was Sie wirklich bekommen</t>
+          <t>Was Sie wirklich erhalten</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Ce que vous obtenez réellement</t>
         </is>
       </c>
       <c r="G55" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Wat U Daadwerkelijk Krijgt</t>
         </is>
       </c>
       <c r="H55" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>您实际获得的</t>
         </is>
       </c>
       <c r="I55" s="6" t="inlineStr">
@@ -3930,23 +4011,26 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Nicht Beratung.
+          <t>Nicht beratend.
 Produktion.</t>
         </is>
       </c>
       <c r="F56" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Pas du conseil.
+De la production.</t>
         </is>
       </c>
       <c r="G56" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Geen advies.
+Productie.</t>
         </is>
       </c>
       <c r="H56" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>不是咨询建议。
+而是生产成果。</t>
         </is>
       </c>
       <c r="I56" s="6" t="inlineStr">
@@ -3985,22 +4069,22 @@
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>Jedes Projekt erzeugt eine Reihe verbundener Outputs, die zusammen definieren, wie Ihr Geschäft als System funktioniert.</t>
+          <t>Jedes Engagement produziert eine Reihe verbundener Outputs, die zusammen definieren, wie Ihr Unternehmen als System funktioniert.</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Chaque engagement produit un ensemble de résultats connectés qui définissent ensemble comment votre entreprise fonctionne en tant que système.</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Elke samenwerking produceert een set verbonden resultaten die tezamen definiëren hoe uw bedrijf als een systeem werkt.</t>
         </is>
       </c>
       <c r="H57" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>每次合作都产生一套相互关联的成果，共同定义您的业务如何作为一个系统运作。</t>
         </is>
       </c>
       <c r="I57" s="6" t="inlineStr">
@@ -4042,17 +4126,17 @@
       </c>
       <c r="F58" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>La hiérarchie est la source de vérité. Tout le reste en est une projection.</t>
         </is>
       </c>
       <c r="G58" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>De hiërarchie is de bron van waarheid. Al het overige is een projectie ervan.</t>
         </is>
       </c>
       <c r="H58" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>层级是事实的唯一来源，其他一切都是它的投影。</t>
         </is>
       </c>
       <c r="I58" s="6" t="inlineStr">
@@ -4094,17 +4178,17 @@
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Résultat 01 — Carte des capacités</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Resultaat 01 — Capability Map</t>
         </is>
       </c>
       <c r="H59" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>成果 01 — 能力地图</t>
         </is>
       </c>
       <c r="I59" s="6" t="inlineStr">
@@ -4141,22 +4225,22 @@
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Definition der Geschäftsmaschine</t>
+          <t>Business-Engine-Definition</t>
         </is>
       </c>
       <c r="F60" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Définition du moteur commercial</t>
         </is>
       </c>
       <c r="G60" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Bedrijfsmotor Definitie</t>
         </is>
       </c>
       <c r="H60" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>业务引擎定义</t>
         </is>
       </c>
       <c r="I60" s="6" t="inlineStr">
@@ -4198,17 +4282,17 @@
       </c>
       <c r="F61" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Résultat 02 — Architecture de flux</t>
         </is>
       </c>
       <c r="G61" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Resultaat 02 — Workflow Architecture</t>
         </is>
       </c>
       <c r="H61" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>成果 02 — 工作流架构</t>
         </is>
       </c>
       <c r="I61" s="6" t="inlineStr">
@@ -4250,17 +4334,17 @@
       </c>
       <c r="F62" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Conception des processus et de l'autorité</t>
         </is>
       </c>
       <c r="G62" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Proces &amp; Autoriteit Ontwerp</t>
         </is>
       </c>
       <c r="H62" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>流程与权限设计</t>
         </is>
       </c>
       <c r="I62" s="6" t="inlineStr">
@@ -4292,7 +4376,22 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Systemlogik-Design</t>
+          <t>System-Logic-Design</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>Conception de la logique système</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>System Logic Ontwerp</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>系统逻辑设计</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -4334,17 +4433,17 @@
       </c>
       <c r="F64" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Spécification de construction (PRD)</t>
         </is>
       </c>
       <c r="G64" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Build Specification (PRD)</t>
         </is>
       </c>
       <c r="H64" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>构建规范（PRD）</t>
         </is>
       </c>
       <c r="I64" s="6" t="inlineStr">
@@ -4381,22 +4480,22 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>KPIs und Observability-Design</t>
+          <t>KPIs und Observability Design</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Conception des KPI et de l'observabilité</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>KPI's &amp; Observability Ontwerp</t>
         </is>
       </c>
       <c r="H65" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>KPI 与可观测性设计</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
@@ -4433,22 +4532,22 @@
       </c>
       <c r="E66" s="6" t="inlineStr">
         <is>
-          <t>Maschinenlesbarer Systemspec</t>
+          <t>Maschinenlesbares Systemspez</t>
         </is>
       </c>
       <c r="F66" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Spécification système consommable par machine</t>
         </is>
       </c>
       <c r="G66" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Machine-Consumable System Spec</t>
         </is>
       </c>
       <c r="H66" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>机器可读系统规范</t>
         </is>
       </c>
       <c r="I66" s="6" t="inlineStr">
@@ -4485,22 +4584,22 @@
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>Für die meisten Teams ist es das erste Mal, dass das Geschäft zu etwas wird, das tatsächlich getestet und durchdacht werden kann.</t>
+          <t>Für die meisten Teams ist es das erste Mal, dass das Unternehmen zu etwas wird, das tatsächlich getestet und durchdacht werden kann.</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Pour la plupart des équipes, c'est la première fois que l'entreprise devient quelque chose qui peut réellement être testé et analysé.</t>
         </is>
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Voor de meeste teams is het de eerste keer dat het bedrijf iets wordt dat daadwerkelijk kan worden getest en redenering kan worden toegepast.</t>
         </is>
       </c>
       <c r="H67" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>对大多数团队而言，这是业务第一次成为可以真正测试和推理的东西。</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -4556,17 +4655,17 @@
       </c>
       <c r="F70" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Étude de cas phare</t>
         </is>
       </c>
       <c r="G70" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Flagship Casestudy</t>
         </is>
       </c>
       <c r="H70" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>旗舰案例研究</t>
         </is>
       </c>
       <c r="I70" s="6" t="inlineStr">
@@ -4603,22 +4702,22 @@
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>Gestaltung eines 1-Milliarden-Dollar-Genetik-Geschäftssystems</t>
+          <t>Gestaltung eines $1B-Genetik-Geschäftssystems</t>
         </is>
       </c>
       <c r="F71" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Conception d'un système commercial en génétique d'un milliard de dollars</t>
         </is>
       </c>
       <c r="G71" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Het ontwerpen van een $1B Genetica Bedrijfssysteem</t>
         </is>
       </c>
       <c r="H71" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>设计一个 10 亿美元遗传学业务系统</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
@@ -4655,22 +4754,22 @@
       </c>
       <c r="E72" s="6" t="inlineStr">
         <is>
-          <t>Wie eine komplexe, mehrakteurige Healthcare-Plattform strukturiert wurde, um zu skalieren — bevor das Volumen ihre Schwächen enthüllte.</t>
+          <t>Wie eine komplexe, Multi-Actor-Healthcare-Plattform strukturiert wurde, um zu skalieren — bevor Volumen ihre Schwächen offenbarte.</t>
         </is>
       </c>
       <c r="F72" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Comment une plateforme de soins de santé complexe et multi-acteurs a été structurée pour évoluer — avant que le volume n'expose ses faiblesses.</t>
         </is>
       </c>
       <c r="G72" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Hoe een complex, multi-actor gezondheidszorgplatform werd gestructureerd om te schalen — voordat volume haar zwakten blootlegde.</t>
         </is>
       </c>
       <c r="H72" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>一个复杂的多方参与医疗保健平台如何被结构化以实现扩展——在流量暴露其弱点之前。</t>
         </is>
       </c>
       <c r="I72" s="6" t="inlineStr">
@@ -4707,22 +4806,22 @@
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>Das System skalierte, weil es zum Funktionieren entworfen wurde — nicht weil es iterativ in Form gebracht wurde.</t>
+          <t>Das System skalierte, weil es funktionieren sollte — nicht weil es in Form iteriert wurde.</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Le système a évolué parce qu'il a été conçu pour fonctionner — non pas parce qu'il a été itéré jusqu'à prendre forme.</t>
         </is>
       </c>
       <c r="G73" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Het systeem schaalde omdat het was ontworpen om te werken — niet omdat het in vorm werd geïtereerd.</t>
         </is>
       </c>
       <c r="H73" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>该系统之所以扩展，是因为它被设计成可运行的——而非通过迭代被塑造成可运行的。</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -4766,22 +4865,22 @@
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>Für wen dies ist</t>
+          <t>Wer das ist</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>À qui c'est destiné</t>
         </is>
       </c>
       <c r="G75" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Voor Wie Dit Is</t>
         </is>
       </c>
       <c r="H75" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>这是为谁准备的</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr">
@@ -4813,7 +4912,22 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Entwickelt für Gründer, Betreiber und Investoren, die in Systemen denken.</t>
+          <t>Gebaut für Gründer, Betreiber und Investoren, die in Systemen denken.</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Construit pour les fondateurs, opérateurs et investisseurs qui pensent en systèmes.</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Gebouwd voor ondernemers, operators en investeerders die in systemen denken.</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>为以系统思维思考的创始人、运营者和投资者而生。</t>
         </is>
       </c>
       <c r="I76" t="inlineStr">
@@ -4855,17 +4969,17 @@
       </c>
       <c r="F77" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Fondateurs</t>
         </is>
       </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Ondernemers</t>
         </is>
       </c>
       <c r="H77" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>创始人</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
@@ -4902,22 +5016,22 @@
       </c>
       <c r="E78" s="6" t="inlineStr">
         <is>
-          <t>Wandeln Sie Ideen in strukturierte, baubare Systeme um. Bauen Sie das richtige Geschäft, nicht nur schnelle Software.</t>
+          <t>Verwandeln Sie Ideen in strukturierte, baubare Systeme. Bauen Sie das richtige Unternehmen, nicht nur schnelle Software.</t>
         </is>
       </c>
       <c r="F78" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Transformez les idées en systèmes structurés et constructibles. Construisez la bonne entreprise, pas juste un logiciel rapide.</t>
         </is>
       </c>
       <c r="G78" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Zet ideeën om in gestructureerde, bouwbare systemen. Bouw het juiste bedrijf, niet alleen snelle software.</t>
         </is>
       </c>
       <c r="H78" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>将创意转化为结构化、可构建的系统。构建正确的业务，而非仅仅快速软件。</t>
         </is>
       </c>
       <c r="I78" s="6" t="inlineStr">
@@ -4954,22 +5068,22 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Operatoren</t>
+          <t>Betreiber</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Opérateurs</t>
         </is>
       </c>
       <c r="G79" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Operators</t>
         </is>
       </c>
       <c r="H79" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>运营者</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -5011,17 +5125,17 @@
       </c>
       <c r="F80" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Investisseurs et capital-investissement</t>
         </is>
       </c>
       <c r="G80" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Investeerders &amp; PE</t>
         </is>
       </c>
       <c r="H80" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>投资者与私募股权</t>
         </is>
       </c>
       <c r="I80" s="6" t="inlineStr">
@@ -5070,17 +5184,17 @@
       </c>
       <c r="F82" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Comment nous travaillons</t>
         </is>
       </c>
       <c r="G82" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Hoe We Werken</t>
         </is>
       </c>
       <c r="H82" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>我们的工作方式</t>
         </is>
       </c>
       <c r="I82" s="6" t="inlineStr">
@@ -5124,17 +5238,20 @@
       </c>
       <c r="F83" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Commencez n'importe où.
+Allez aussi loin que vous le souhaitez.</t>
         </is>
       </c>
       <c r="G83" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Begin overal.
+Ga zo ver als u nodig hebt.</t>
         </is>
       </c>
       <c r="H83" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>从任何地方开始。
+根据需要深入推进。</t>
         </is>
       </c>
       <c r="I83" s="6" t="inlineStr">
@@ -5178,17 +5295,17 @@
       </c>
       <c r="F84" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>La plupart de nos clients commencent par une seule séance. Aucun engagement au-delà de cela.</t>
         </is>
       </c>
       <c r="G84" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>De meeste klanten beginnen met een enkele sessie. Geen verplichting voorbij dat.</t>
         </is>
       </c>
       <c r="H84" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>大多数客户从一次会议开始，没有超越此外的承诺。</t>
         </is>
       </c>
       <c r="I84" s="6" t="inlineStr">
@@ -5223,6 +5340,21 @@
           <t>Discovery-Sitzung</t>
         </is>
       </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Séance de découverte</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Discovery Session</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>发现会议</t>
+        </is>
+      </c>
       <c r="I85" t="inlineStr">
         <is>
           <t>Phiên Khám phá</t>
@@ -5257,22 +5389,22 @@
       </c>
       <c r="E86" s="6" t="inlineStr">
         <is>
+          <t>GEARS™ System-Design</t>
+        </is>
+      </c>
+      <c r="F86" s="6" t="inlineStr">
+        <is>
+          <t>Conception de système GEARS™</t>
+        </is>
+      </c>
+      <c r="G86" s="6" t="inlineStr">
+        <is>
           <t>GEARS™ System Design</t>
         </is>
       </c>
-      <c r="F86" s="6" t="inlineStr">
-        <is>
-          <t>— TO BE TRANSLATED —</t>
-        </is>
-      </c>
-      <c r="G86" s="6" t="inlineStr">
-        <is>
-          <t>— TO BE TRANSLATED —</t>
-        </is>
-      </c>
       <c r="H86" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GEARS™ 系统设计</t>
         </is>
       </c>
       <c r="I86" s="6" t="inlineStr">
@@ -5309,22 +5441,22 @@
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
+          <t>Build-Partnerschaft</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>Partenariat de construction</t>
+        </is>
+      </c>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
           <t>Build Partnership</t>
         </is>
       </c>
-      <c r="F87" s="6" t="inlineStr">
-        <is>
-          <t>— TO BE TRANSLATED —</t>
-        </is>
-      </c>
-      <c r="G87" s="6" t="inlineStr">
-        <is>
-          <t>— TO BE TRANSLATED —</t>
-        </is>
-      </c>
       <c r="H87" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>构建合作伙伴关系</t>
         </is>
       </c>
       <c r="I87" s="6" t="inlineStr">
@@ -5361,22 +5493,22 @@
       </c>
       <c r="E88" s="6" t="inlineStr">
         <is>
-          <t>Betreiben &amp; Weiterentwickeln</t>
+          <t>Betreiben &amp; Entwickeln</t>
         </is>
       </c>
       <c r="F88" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Opérer et évoluer</t>
         </is>
       </c>
       <c r="G88" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Bedrijfsvoering &amp; Evolutie</t>
         </is>
       </c>
       <c r="H88" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>运营与演进</t>
         </is>
       </c>
       <c r="I88" s="6" t="inlineStr">
@@ -5411,6 +5543,21 @@
           <t>Sitzung buchen</t>
         </is>
       </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Réservez une séance</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Boek een sessie</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>预约会议</t>
+        </is>
+      </c>
       <c r="I89" t="inlineStr">
         <is>
           <t>Đặt lịch phiên</t>
@@ -5452,22 +5599,22 @@
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>Vertraut von Operatoren</t>
+          <t>Vertraut von Betreibern</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Approuvé par les opérateurs</t>
         </is>
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Vertrouwd door Operators</t>
         </is>
       </c>
       <c r="H91" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>值得信赖的运营者</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
@@ -5504,22 +5651,22 @@
       </c>
       <c r="E92" s="6" t="inlineStr">
         <is>
-          <t>"GKIM hat mir geholfen, meine Vision zu entwickeln und sie in ein durchdachtes Geschäfts-, Produkt- und Technologieangebot umzuwandeln. Das Team hat sich bei der Umsetzung hervorgetan."</t>
+          <t>"GKIM hat mir geholfen, meine Vision zu ideensammeln und sie in ein durchdachtes Unternehmen, Produkt und Technologieangebot umzuwandeln. Das Team hat bei der Umsetzung hervorragende Leistungen erbracht."</t>
         </is>
       </c>
       <c r="F92" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>« GKIM m'a aidé à réfléchir à ma vision et à la transformer en une offre commerciale, produit et technologie bien pensée. L'équipe a excellé dans l'exécution. »</t>
         </is>
       </c>
       <c r="G92" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>"GKIM hielp bij het brainstormen van mijn visie en het opbouwen ervan in een goed doordacht bedrijfs-, product- en technologie-aanbod. Het team heeft zich uitstekend ingespannen bij de uitvoering."</t>
         </is>
       </c>
       <c r="H92" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>"GKIM 帮助我将愿景头脑风暴并将其构建成经过深思熟虑的业务、产品和技术方案。该团队在执行方面表现出色。"</t>
         </is>
       </c>
       <c r="I92" s="6" t="inlineStr">
@@ -5561,17 +5708,17 @@
       </c>
       <c r="F93" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Fondateur et PDG</t>
         </is>
       </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Oprichter &amp; CEO</t>
         </is>
       </c>
       <c r="H93" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>创始人兼首席执行官</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
@@ -5622,22 +5769,22 @@
       </c>
       <c r="E96" s="6" t="inlineStr">
         <is>
-          <t>Gebaut von jemandem, der dies schon einmal getan hat</t>
+          <t>Gebaut von jemandem, der dies schon getan hat</t>
         </is>
       </c>
       <c r="F96" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Construit par quelqu'un qui a déjà fait cela</t>
         </is>
       </c>
       <c r="G96" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Gebouwd door Iemand Die Dit Eerder Heeft Gedaan</t>
         </is>
       </c>
       <c r="H96" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>由有过此经验的人创建</t>
         </is>
       </c>
       <c r="I96" s="6" t="inlineStr">
@@ -5674,22 +5821,22 @@
       </c>
       <c r="E97" s="6" t="inlineStr">
         <is>
-          <t>An die Gründer und Führungskräfte, die die Zukunft gestalten,</t>
+          <t>An die Gründer und Führungskräfte, die die Zukunft bauen,</t>
         </is>
       </c>
       <c r="F97" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Aux fondateurs et aux leaders qui construisent l'avenir,</t>
         </is>
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Aan de Oprichters en Leiders die de Toekomst Bouwen,</t>
         </is>
       </c>
       <c r="H97" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>致正在打造未来的创始人和领导者，</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
@@ -5731,17 +5878,17 @@
       </c>
       <c r="F98" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>— Ian Morrison</t>
         </is>
       </c>
       <c r="G98" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>— Ian Morrison</t>
         </is>
       </c>
       <c r="H98" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>— Ian Morrison</t>
         </is>
       </c>
       <c r="I98" s="6" t="inlineStr">
@@ -5783,17 +5930,17 @@
       </c>
       <c r="F99" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Ce qui rend GKIM différent</t>
         </is>
       </c>
       <c r="G99" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Wat Maakt GKIM Anders</t>
         </is>
       </c>
       <c r="H99" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>是什么使 GKIM 与众不同</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
@@ -5842,17 +5989,17 @@
       </c>
       <c r="F101" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Parlez à GKIM</t>
         </is>
       </c>
       <c r="G101" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Neem Contact Op Met GKIM</t>
         </is>
       </c>
       <c r="H101" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>联系 GKIM</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -5889,22 +6036,22 @@
       </c>
       <c r="E102" s="6" t="inlineStr">
         <is>
-          <t>Bevor Sie bauen oder skalieren, verstehen Sie, wie Ihr Geschäft tatsächlich funktioniert.</t>
+          <t>Bevor Sie bauen oder skalieren, verstehen Sie, wie Ihr Unternehmen wirklich funktioniert.</t>
         </is>
       </c>
       <c r="F102" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Avant de construire ou de développer, comprenez comment votre entreprise fonctionne réellement.</t>
         </is>
       </c>
       <c r="G102" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Voordat u bouwt of schaalt, begrijpt u hoe uw bedrijf daadwerkelijk werkt.</t>
         </is>
       </c>
       <c r="H102" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>在构建或扩展前，了解您的业务实际运作方式。</t>
         </is>
       </c>
       <c r="I102" s="6" t="inlineStr">
@@ -5946,17 +6093,17 @@
       </c>
       <c r="F103" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Ce n'est pas un appel de vente. C'est une séance de travail pour comprendre votre modèle commercial, explorer comment le système fonctionne actuellement, et identifier les lacunes, les risques et les hypothèses.</t>
         </is>
       </c>
       <c r="G103" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Dit is geen verkoopgesprek. Het is een werkzitting om uw bedrijfsmodel te begrijpen, de huidige werking van het systeem te onderzoeken en hiaten, risico's en aannames te identificeren.</t>
         </is>
       </c>
       <c r="H103" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>这不是销售电话，而是一次工作会议，旨在了解您的商业模式，探索系统当前的运作方式，并识别差距、风险和假设。</t>
         </is>
       </c>
       <c r="I103" s="6" t="inlineStr">
@@ -5993,22 +6140,22 @@
       </c>
       <c r="E104" s="6" t="inlineStr">
         <is>
-          <t>Klarheit ersetzt Annahmen.</t>
+          <t>Klarheit ersetzt Annahme.</t>
         </is>
       </c>
       <c r="F104" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>La clarté remplace l'hypothèse.</t>
         </is>
       </c>
       <c r="G104" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Helderheid vervangt aanname.</t>
         </is>
       </c>
       <c r="H104" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>清晰取代假设。</t>
         </is>
       </c>
       <c r="I104" s="6" t="inlineStr">
@@ -6045,22 +6192,22 @@
       </c>
       <c r="E105" s="6" t="inlineStr">
         <is>
-          <t>Erzählen Sie uns, was Sie bauen, wo Sie sich auf der Reise befinden und was unklar oder nicht funktionierend wirkt.</t>
+          <t>Sagen Sie uns, was Sie bauen, wo Sie sich auf der Reise befinden und was unklar oder nicht funktionierend wirkt.</t>
         </is>
       </c>
       <c r="F105" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Dites-nous ce que vous construisez, où vous en êtes dans le parcours, et ce qui vous semble peu clair ou ne fonctionne pas.</t>
         </is>
       </c>
       <c r="G105" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Vertel ons wat u bouwt, waar u zich in de reis bevindt en wat onduidelijk is of niet werkt.</t>
         </is>
       </c>
       <c r="H105" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>告诉我们您正在构建什么，您在历程中处于何位置，以及什么感觉不清楚或不起作用。</t>
         </is>
       </c>
       <c r="I105" s="6" t="inlineStr">
@@ -6112,7 +6259,7 @@
       </c>
       <c r="H106" s="2" t="inlineStr">
         <is>
-          <t>姓名</t>
+          <t>名字</t>
         </is>
       </c>
       <c r="I106" s="2" t="inlineStr">
@@ -6147,6 +6294,21 @@
           <t>Unternehmen</t>
         </is>
       </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>Entreprise</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Bedrijf</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>公司</t>
+        </is>
+      </c>
       <c r="I107" t="inlineStr">
         <is>
           <t>Công ty</t>
@@ -6196,7 +6358,7 @@
       </c>
       <c r="H108" s="2" t="inlineStr">
         <is>
-          <t>邮箱</t>
+          <t>电子邮件</t>
         </is>
       </c>
       <c r="I108" s="2" t="inlineStr">
@@ -6238,17 +6400,17 @@
       </c>
       <c r="F109" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Qu'êtes-vous en train de construire ou qu'est-ce qui ne fonctionne pas ?</t>
         </is>
       </c>
       <c r="G109" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Wat bouwt u of wat werkt niet?</t>
         </is>
       </c>
       <c r="H109" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>您在构建什么或什么不起作用？</t>
         </is>
       </c>
       <c r="I109" s="6" t="inlineStr">
@@ -6290,17 +6452,17 @@
       </c>
       <c r="F110" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Partagez autant ou aussi peu que vous le souhaitez...</t>
         </is>
       </c>
       <c r="G110" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Deel zoveel of zo weinig als je wilt...</t>
         </is>
       </c>
       <c r="H110" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>尽可能多或少地分享……</t>
         </is>
       </c>
       <c r="I110" s="6" t="inlineStr">
@@ -6342,17 +6504,17 @@
       </c>
       <c r="F111" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Réservez une séance</t>
         </is>
       </c>
       <c r="G111" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Boek een Sessie</t>
         </is>
       </c>
       <c r="H111" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>预约会议</t>
         </is>
       </c>
       <c r="I111" s="6" t="inlineStr">
@@ -6396,22 +6558,22 @@
       </c>
       <c r="E113" s="6" t="inlineStr">
         <is>
-          <t>Gestalten Sie das Geschäft, bevor Sie es bauen</t>
+          <t>Gestalten Sie das Unternehmen, bevor Sie es bauen</t>
         </is>
       </c>
       <c r="F113" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Concevez l'entreprise avant de la construire</t>
         </is>
       </c>
       <c r="G113" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Ontwerp het bedrijf voordat u het bouwt</t>
         </is>
       </c>
       <c r="H113" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>在构建前设计业务</t>
         </is>
       </c>
       <c r="I113" s="6" t="inlineStr">
@@ -6453,17 +6615,17 @@
       </c>
       <c r="F114" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>La plupart des équipes commencent par le code. Les meilleures équipes commencent par la clarté.</t>
         </is>
       </c>
       <c r="G114" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>De meeste teams beginnen met code. De beste teams beginnen met helderheid.</t>
         </is>
       </c>
       <c r="H114" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>大多数团队从代码开始，最好的团队从清晰开始。</t>
         </is>
       </c>
       <c r="I114" s="6" t="inlineStr">
@@ -6505,17 +6667,17 @@
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
-          <t>Discutons</t>
+          <t>Parlez à GKIM</t>
         </is>
       </c>
       <c r="G115" s="2" t="inlineStr">
         <is>
-          <t>Contact opnemen</t>
+          <t>Neem contact op met GKIM</t>
         </is>
       </c>
       <c r="H115" s="2" t="inlineStr">
         <is>
-          <t>联系我们</t>
+          <t>联系 GKIM</t>
         </is>
       </c>
       <c r="I115" s="2" t="inlineStr">
@@ -6606,7 +6768,22 @@
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>Gestalten Sie Ihr KI-natives Geschäft.</t>
+          <t>Gestalten Sie Ihr KI-natives Unternehmen.</t>
+        </is>
+      </c>
+      <c r="F118" t="inlineStr">
+        <is>
+          <t>Concevez votre entreprise native IA.</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Ontwerp uw AI-native bedrijf.</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr">
+        <is>
+          <t>设计您的 AI 原生业务。</t>
         </is>
       </c>
       <c r="I118" t="inlineStr">
@@ -6648,17 +6825,17 @@
       </c>
       <c r="F119" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Explorer</t>
         </is>
       </c>
       <c r="G119" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Verkennen</t>
         </is>
       </c>
       <c r="H119" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>探索</t>
         </is>
       </c>
       <c r="I119" s="6" t="inlineStr">
@@ -6700,17 +6877,17 @@
       </c>
       <c r="F120" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="G120" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="H120" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>联系</t>
         </is>
       </c>
       <c r="I120" s="6" t="inlineStr">
@@ -6799,22 +6976,22 @@
       </c>
       <c r="E122" s="6" t="inlineStr">
         <is>
-          <t>Systemdefinition. KI-natives Business Design.</t>
+          <t>System-Definition. KI-natives Business-Design.</t>
         </is>
       </c>
       <c r="F122" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>Définition du système. Conception d'entreprise native IA.</t>
         </is>
       </c>
       <c r="G122" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>System definitie. AI-native bedrijfsontwerp.</t>
         </is>
       </c>
       <c r="H122" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>系统定义。AI 原生业务设计。</t>
         </is>
       </c>
       <c r="I122" s="6" t="inlineStr">
@@ -6858,22 +7035,22 @@
       </c>
       <c r="E124" s="6" t="inlineStr">
         <is>
-          <t>GKIM Digital — Gestalten Sie Ihr KI-natives Geschäft</t>
+          <t>GKIM Digital — Gestalten Sie Ihr KI-natives Unternehmen</t>
         </is>
       </c>
       <c r="F124" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GKIM Digital — Concevez votre entreprise native IA</t>
         </is>
       </c>
       <c r="G124" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GKIM Digital — Ontwerp Uw AI-Native Bedrijf</t>
         </is>
       </c>
       <c r="H124" s="6" t="inlineStr">
         <is>
-          <t>— TO BE TRANSLATED —</t>
+          <t>GKIM Digital — 设计您的 AI 原生业务</t>
         </is>
       </c>
       <c r="I124" s="6" t="inlineStr">
@@ -6915,7 +7092,7 @@
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
-          <t>fr</t>
+          <t>en</t>
         </is>
       </c>
       <c r="G125" s="2" t="inlineStr">
@@ -6925,7 +7102,7 @@
       </c>
       <c r="H125" s="2" t="inlineStr">
         <is>
-          <t>zh-Hans</t>
+          <t>zh</t>
         </is>
       </c>
       <c r="I125" s="2" t="inlineStr">
@@ -6965,8 +7142,29 @@
       <c r="E126" t="inlineStr">
         <is>
           <t>GKIM Papers —
-Originäres Denken über
-KI-native Geschäftsmodelle</t>
+Originalgedanken zu
+KI-nativem Business-Design</t>
+        </is>
+      </c>
+      <c r="F126" t="inlineStr">
+        <is>
+          <t>Documents GKIM —
+Réflexion originale sur
+la conception d'entreprise native IA</t>
+        </is>
+      </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>GKIM Papers —
+Origineel denken over
+AI-native bedrijfsontwerp</t>
+        </is>
+      </c>
+      <c r="H126" t="inlineStr">
+        <is>
+          <t>GKIM 论文 —
+关于 AI 原生业务设计的
+原创思考</t>
         </is>
       </c>
       <c r="I126" t="inlineStr">
@@ -7002,7 +7200,22 @@
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>Fünfzehn Papiere über fünf Themen. Geschrieben für Gründer, Operatoren und Investoren, die die Architektur der kommenden Entwicklungen verstehen möchten.</t>
+          <t>Fünfzehn Papiere in fünf Themen. Geschrieben für Gründer, Betreiber und Investoren, die die Architektur der kommenden Zukunft verstehen möchten.</t>
+        </is>
+      </c>
+      <c r="F127" t="inlineStr">
+        <is>
+          <t>Quinze documents sur cinq thèmes. Rédigés pour les fondateurs, opérateurs et investisseurs qui souhaitent comprendre l'architecture de ce qui arrive.</t>
+        </is>
+      </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>Vijftien papers over vijf thema's. Geschreven voor ondernemers, operators en investeerders die de architectuur van wat eraan komt willen begrijpen.</t>
+        </is>
+      </c>
+      <c r="H127" t="inlineStr">
+        <is>
+          <t>跨越五个主题的十五篇论文。为希望理解未来架构的创始人、运营者和投资者而写。</t>
         </is>
       </c>
       <c r="I127" t="inlineStr">
@@ -7042,6 +7255,21 @@
           <t>Grundlagen</t>
         </is>
       </c>
+      <c r="F128" t="inlineStr">
+        <is>
+          <t>Fondations</t>
+        </is>
+      </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>Fundamenten</t>
+        </is>
+      </c>
+      <c r="H128" t="inlineStr">
+        <is>
+          <t>基础</t>
+        </is>
+      </c>
       <c r="I128" t="inlineStr">
         <is>
           <t>Nền tảng</t>
@@ -7076,7 +7304,22 @@
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>Was ist ein KI-natives Geschäftsmodell?</t>
+          <t>Was ist ein KI-natives Unternehmen?</t>
+        </is>
+      </c>
+      <c r="F129" t="inlineStr">
+        <is>
+          <t>Qu'est-ce qu'une entreprise native IA ?</t>
+        </is>
+      </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>Wat is een AI-Native Bedrijf?</t>
+        </is>
+      </c>
+      <c r="H129" t="inlineStr">
+        <is>
+          <t>什么是 AI 原生业务？</t>
         </is>
       </c>
       <c r="I129" t="inlineStr">
@@ -7116,6 +7359,21 @@
           <t>3 Papiere</t>
         </is>
       </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>3 documents</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr">
+        <is>
+          <t>3 篇论文</t>
+        </is>
+      </c>
       <c r="I130" t="inlineStr">
         <is>
           <t>3 bài viết</t>
@@ -7150,7 +7408,22 @@
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Das Argument dafür</t>
+          <t>Die Argumentation</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>L'argument en faveur</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Het Geval Voor</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr">
+        <is>
+          <t>支持理由</t>
         </is>
       </c>
       <c r="I131" t="inlineStr">
@@ -7187,7 +7460,22 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>Das strategische und ökonomische Argument</t>
+          <t>Das strategische und wirtschaftliche Argument</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>L'argument stratégique et économique</t>
+        </is>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>Het Strategische &amp; Economische Argument</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr">
+        <is>
+          <t>战略与经济论证</t>
         </is>
       </c>
       <c r="I132" t="inlineStr">
@@ -7222,6 +7510,21 @@
           <t>3 Papiere</t>
         </is>
       </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>3 documents</t>
+        </is>
+      </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="H133" t="inlineStr">
+        <is>
+          <t>3 篇论文</t>
+        </is>
+      </c>
       <c r="I133" t="inlineStr">
         <is>
           <t>3 bài viết</t>
@@ -7256,7 +7559,22 @@
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>Vertrauen und Sicherheit</t>
+          <t>Vertrauen &amp; Sicherheit</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>Confiance et sécurité</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>Vertrouwen &amp; Veiligheid</t>
+        </is>
+      </c>
+      <c r="H134" t="inlineStr">
+        <is>
+          <t>信任与安全</t>
         </is>
       </c>
       <c r="I134" t="inlineStr">
@@ -7293,7 +7611,22 @@
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>Governance, Menschen und Verantwortung</t>
+          <t>Governance, Menschen &amp; Rechenschaftspflicht</t>
+        </is>
+      </c>
+      <c r="F135" t="inlineStr">
+        <is>
+          <t>Gouvernance, humains et responsabilité</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>Governance, Mensen &amp; Accountability</t>
+        </is>
+      </c>
+      <c r="H135" t="inlineStr">
+        <is>
+          <t>治理、人员与问责</t>
         </is>
       </c>
       <c r="I135" t="inlineStr">
@@ -7328,6 +7661,21 @@
           <t>3 Papiere</t>
         </is>
       </c>
+      <c r="F136" t="inlineStr">
+        <is>
+          <t>3 documents</t>
+        </is>
+      </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="H136" t="inlineStr">
+        <is>
+          <t>3 篇论文</t>
+        </is>
+      </c>
       <c r="I136" t="inlineStr">
         <is>
           <t>3 bài viết</t>
@@ -7362,7 +7710,22 @@
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>Playbook für Gründer</t>
+          <t>Gründer-Playbook</t>
+        </is>
+      </c>
+      <c r="F137" t="inlineStr">
+        <is>
+          <t>Playbook des fondateurs</t>
+        </is>
+      </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>Oprichtersplaybook</t>
+        </is>
+      </c>
+      <c r="H137" t="inlineStr">
+        <is>
+          <t>创始人手册</t>
         </is>
       </c>
       <c r="I137" t="inlineStr">
@@ -7402,6 +7765,21 @@
           <t>Praktische Überzeugung für Builder</t>
         </is>
       </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>Conviction pratique pour les constructeurs</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>Praktische Overtuiging voor Bouwers</t>
+        </is>
+      </c>
+      <c r="H138" t="inlineStr">
+        <is>
+          <t>构建者的实用信念</t>
+        </is>
+      </c>
       <c r="I138" t="inlineStr">
         <is>
           <t>Quyết tâm thực tiễn cho những người xây dựng</t>
@@ -7434,6 +7812,21 @@
           <t>3 Papiere</t>
         </is>
       </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>3 documents</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="H139" t="inlineStr">
+        <is>
+          <t>3 篇论文</t>
+        </is>
+      </c>
       <c r="I139" t="inlineStr">
         <is>
           <t>3 bài viết</t>
@@ -7468,7 +7861,22 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Architektur und Lebenszyklus</t>
+          <t>Architektur &amp; Lebenszyklus</t>
+        </is>
+      </c>
+      <c r="F140" t="inlineStr">
+        <is>
+          <t>Architecture et cycle de vie</t>
+        </is>
+      </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>Architectuur &amp; Levenscyclus</t>
+        </is>
+      </c>
+      <c r="H140" t="inlineStr">
+        <is>
+          <t>架构与生命周期</t>
         </is>
       </c>
       <c r="I140" t="inlineStr">
@@ -7505,7 +7913,22 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Wie diese Geschäftsmodelle aufgebaut sind</t>
+          <t>Wie diese Unternehmen gebaut werden</t>
+        </is>
+      </c>
+      <c r="F141" t="inlineStr">
+        <is>
+          <t>Comment ces entreprises sont construites</t>
+        </is>
+      </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>Hoe Deze Bedrijven Worden Gebouwd</t>
+        </is>
+      </c>
+      <c r="H141" t="inlineStr">
+        <is>
+          <t>这些业务如何被构建</t>
         </is>
       </c>
       <c r="I141" t="inlineStr">
@@ -7540,6 +7963,21 @@
           <t>3 Papiere</t>
         </is>
       </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>3 documents</t>
+        </is>
+      </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>3 papers</t>
+        </is>
+      </c>
+      <c r="H142" t="inlineStr">
+        <is>
+          <t>3 篇论文</t>
+        </is>
+      </c>
       <c r="I142" t="inlineStr">
         <is>
           <t>3 bài viết</t>
@@ -7574,7 +8012,22 @@
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>Jedes Papier dauert 7–11 Minuten zum Lesen. Vollständige PDFs folgen in Kürze. Geschrieben aus Cambridge — nicht von einer Konferenzbühne.</t>
+          <t>Jedes Papier dauert 7–11 Minuten. Vollständige PDFs folgen in Kürze. Geschrieben aus Cambridge — nicht von einer Konferenzbühne.</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>Chaque document dure 7 à 11 minutes. Les PDF complets arrivent bientôt. Rédigés de Cambridge — non pas depuis une scène de conférence.</t>
+        </is>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Elk paper is 7–11 minuten. Volledige PDF's binnenkort beschikbaar. Geschreven vanuit Cambridge — niet vanaf een conferentiepodum.</t>
+        </is>
+      </c>
+      <c r="H143" t="inlineStr">
+        <is>
+          <t>每篇论文为 7-11 分钟阅读量。完整 PDF 即将推出。由剑桥撰写——而非来自会议舞台。</t>
         </is>
       </c>
       <c r="I143" t="inlineStr">
@@ -7612,6 +8065,21 @@
       <c r="E144" t="inlineStr">
         <is>
           <t>GKIM Papers lesen →</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>Lire les documents GKIM →</t>
+        </is>
+      </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>Lees GKIM Papers →</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr">
+        <is>
+          <t>阅读 GKIM 论文 →</t>
         </is>
       </c>
       <c r="I144" t="inlineStr">

</xml_diff>

<commit_message>
feat: redesign hero section with new title and subtitle structure
- New h1: "Partnering for success in the AI-native future" (AI-native future in yellow, line break on desktop)
- Old h1 moved to subtitle below the heading
- Body text unchanged

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -1772,7 +1772,7 @@
     <row r="14" ht="36" customHeight="1" s="12">
       <c r="A14" t="inlineStr">
         <is>
-          <t>hero.h1.part1</t>
+          <t>hero.h1.line1</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1782,12 +1782,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Hero h1 — text before the accented phrase</t>
+          <t>Hero h1 — first line</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Your business should</t>
+          <t>Partnering for success in the</t>
         </is>
       </c>
     </row>
@@ -1804,19 +1804,19 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Hero h1 — yellow-highlighted phrase</t>
+          <t>Hero h1 — yellow accented phrase (second line)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>run, learn, and improve</t>
+          <t>AI-native future</t>
         </is>
       </c>
     </row>
     <row r="16" ht="36" customHeight="1" s="12">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hero.h1.part2</t>
+          <t>hero.subtitle</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1826,12 +1826,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Hero h1 — text after the accented phrase</t>
+          <t>Hero subtitle — displayed below the main title</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>on its own.</t>
+          <t>Your business should run, learn, and improve on its own.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update nav, footer, and About page across all pages
- Remove Insights from all nav/footer; simplify nav to GEARS™ · Proof · About + Book a call
- All CTA buttons now link to /discovery/ (removed cal.com links)
- Remove Marketing Systems case study from homepage
- Redesign footer: 5-column layout (logo+socials, Explore, Ian Morrison, UK Office, Vietnam Office)
- Add contact info to footer across all pages (en, about, discovery, confirm)
- Update company LinkedIn link in footer
- Build out About page with full content, team cards, engine room carousel, principles section
- Add team photos for all members

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -952,7 +952,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -999,7 +999,7 @@
       </c>
       <c r="F4" s="6" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
@@ -1093,7 +1093,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>live</t>
+          <t>draft</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Add '04 / The Path' section with three-step timeline to homepage
Inserts a new section between 'The GKIM View' and 'The GEARS Approach'.
Renumbers downstream sections: GEARS→05, Commercial Proof→06, Human Role→07.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -1488,7 +1488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J137"/>
+  <dimension ref="A1:S137"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="12" min="1" max="1"/>
@@ -2922,7 +2922,7 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>04 / The GEARS Approach</t>
+          <t>05 / The GEARS Approach</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>05 / Commercial Proof</t>
+          <t>06 / Commercial Proof</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>06 / The Human Role</t>
+          <t>07 / The Human Role</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Redesign homepage sections: Path, GKIM View, quote; update step content
- Swap order: The Path (03, dark bg) now precedes The GKIM View (04, light bg)
- Remove The GEARS Approach section
- Quote section background changed from yellow to black
- "A design & operating partner" card now has yellow background
- Update step titles and copy in The Path timeline
- Renumber downstream sections: Commercial Proof→05, Human Role→06

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -2695,7 +2695,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>03 / The GKIM View</t>
+          <t>04 / The GKIM View</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3371,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>06 / Commercial Proof</t>
+          <t>05 / Commercial Proof</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>07 / The Human Role</t>
+          <t>06 / The Human Role</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Redesign homepage: interactive Path section, benefits grid, section reorder
- Hero: drop eyebrow, rename Telehealth OS stat to Healthcare OS, update copy
- Shift section: new copy, single-line heading, narrower text column, breakpoint
- Path section: convert to accordion (title + body + matching visual per step),
  embed and brand-recolor three custom SVG illustrations for each step
- Remove "The Problem" section and all numbered eyebrows
- Human Role: move after Path, switch to light background, new copy/CTA text
- Add new Benefits section with branded icon set, single row on desktop
- Reorder Position/GKIM View + quote block relative to Benefits and Proof
</commit_message>
<xml_diff>
--- a/gkim-content.xlsx
+++ b/gkim-content.xlsx
@@ -1488,7 +1488,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S137"/>
+  <dimension ref="A1:J150"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" style="12" min="1" max="1"/>
@@ -1970,7 +1970,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Telehealth OS</t>
+          <t>Healthcare OS</t>
         </is>
       </c>
     </row>
@@ -1992,7 +1992,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>A genetics-led operating system built as integrated business architecture</t>
+          <t>Clinical workflows, compliance and patient engagement, designed as one system</t>
         </is>
       </c>
     </row>
@@ -2036,7 +2036,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Designed from inception, not retrofitted onto legacy operations</t>
+          <t>For businesses starting out, and businesses starting over</t>
         </is>
       </c>
     </row>
@@ -2065,7 +2065,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>01 / The Shift</t>
+          <t>The Shift</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>AI is changing the structure of business,</t>
+          <t>AI is Changing the Structure of Business</t>
         </is>
       </c>
     </row>
@@ -2107,11 +2107,6 @@
           <t>Section heading — second line (after line break on desktop)</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>not just the software.</t>
-        </is>
-      </c>
     </row>
     <row r="31" ht="36" customHeight="1" s="12">
       <c r="A31" t="inlineStr">
@@ -2131,7 +2126,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>For decades, businesses scaled through human coordination: meetings, departments, reporting layers, and fragmented systems. Software accelerated execution, but the business itself stayed hard to design, understand, and evolve.</t>
+          <t>For decades, businesses scaled through human coordination: meetings, departments, reporting layers, and fragmented systems. Software accelerated execution, but the business operation itself stayed hard to evolve.</t>
         </is>
       </c>
     </row>
@@ -2153,7 +2148,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>AI is now compressing the distance between intention and execution.</t>
+          <t>What a business knows has always lived in people's heads and disconnected systems. It can now be captured, modelled, and run.</t>
         </is>
       </c>
     </row>
@@ -2175,7 +2170,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>The companies that win the next decade won't merely use AI tools.</t>
+          <t>The companies that win the next decade will design their businesses</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2192,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>They'll design</t>
+          <t>as</t>
         </is>
       </c>
     </row>
@@ -2239,11 +2234,6 @@
           <t>Large statement — text after the highlighted phrase</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>for their businesses.</t>
-        </is>
-      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -2695,7 +2685,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>04 / The GKIM View</t>
+          <t>The GKIM View</t>
         </is>
       </c>
     </row>
@@ -3371,7 +3361,7 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>05 / Commercial Proof</t>
+          <t>Commercial Proof</t>
         </is>
       </c>
     </row>
@@ -3879,7 +3869,7 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>06 / The Human Role</t>
+          <t>The Human Role</t>
         </is>
       </c>
     </row>
@@ -3901,7 +3891,7 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>This is not about replacing humans.</t>
+          <t>This isn't about replacing your team.</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3913,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>It's about elevating them.</t>
+          <t>It's about accelerating them.</t>
         </is>
       </c>
     </row>
@@ -3945,7 +3935,7 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>AI-native business design removes friction so people can operate at their highest level of contribution. AI expands execution capacity: coordinating workflows, analysing systems, surfacing optimisation, and automating the repetitive. Humans stay where humans matter most.</t>
+          <t>AI-native business removes friction so team can operate at their highest level of contribution. AI expands execution capacity. The work gets more interesting, not less.</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3979,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Humans set the goals and direct strategy</t>
+          <t>You set the goals and direct strategy</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4023,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Humans exercise judgment on what matters</t>
+          <t>You exercise judgment on what matters</t>
         </is>
       </c>
     </row>
@@ -4077,7 +4067,7 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Humans build the relationships that carry value</t>
+          <t>You build the relationships that carry value</t>
         </is>
       </c>
     </row>
@@ -4121,7 +4111,7 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Humans shape the customer value being created</t>
+          <t>You shape the customer value being created</t>
         </is>
       </c>
     </row>
@@ -4165,173 +4155,384 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Humans oversee how the system evolves</t>
+          <t>You oversee how the system evolves</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FINAL CTA</t>
+          <t xml:space="preserve">  BENEFITS</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>cta.eyebrow</t>
+          <t>benefits.eyebrow</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>cta</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Final CTA section eyebrow</t>
+          <t>benefits</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Design the business before you build the software</t>
+          <t>The Benefits</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>cta.h2</t>
+          <t>benefits.h2</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>cta</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>Final CTA heading</t>
+          <t>benefits</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Let's build your AI-native business.</t>
+          <t>What Changes When the Business is AI-Native</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>cta.btn</t>
+          <t>benefits.item1.title</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>cta</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>Final CTA button label</t>
+          <t>benefits</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Book a discovery call</t>
+          <t>Quote faster</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t xml:space="preserve">  FOOTER</t>
+          <t>benefits.item1.desc</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>benefits</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>Because the answer isn't in one person's head.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>footer.tag</t>
+          <t>benefits.item2.title</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>footer</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>Footer tagline below logo</t>
+          <t>benefits</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Designing AI-native business systems through GEARS. Define → Design → Simulate → Build → Operate → Evolve.</t>
+          <t>Grow without hiring behind it</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>footer.proof</t>
+          <t>benefits.item2.desc</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>footer</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>Footer nav link — Commercial Proof section</t>
+          <t>benefits</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Commercial Proof</t>
+          <t>Capacity stops being headcount.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>footer.copy</t>
+          <t>benefits.item3.title</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>footer</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>Footer copyright suffix (after © year)</t>
+          <t>benefits</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>GKIM. All rights reserved.</t>
+          <t>Change the model in a week</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
+          <t>benefits.item3.desc</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>benefits</t>
+        </is>
+      </c>
+      <c r="D137" t="inlineStr">
+        <is>
+          <t>It's documented, not remembered.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>benefits.item4.title</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>benefits</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Improve without a project</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>benefits.item4.desc</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>benefits</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Optimisation is continuous, not quarterly.</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>benefits.item5.title</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>benefits</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>See it live</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>benefits.item5.desc</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>benefits</t>
+        </is>
+      </c>
+      <c r="D141" t="inlineStr">
+        <is>
+          <t>Reporting stops being a person's job.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FINAL CTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>cta.eyebrow</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Final CTA section eyebrow</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Design the business before you build the software</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>cta.h2</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Final CTA heading</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Let's build your AI-native business.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>cta.btn</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>cta</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Final CTA button label</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Book a discovery call</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  FOOTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>footer.tag</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>footer</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Footer tagline below logo</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Designing AI-native business systems through GEARS. Define → Design → Simulate → Build → Operate → Evolve.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>footer.proof</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>footer</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Footer nav link — Commercial Proof section</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Commercial Proof</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>footer.copy</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>footer</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Footer copyright suffix (after © year)</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>GKIM. All rights reserved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
           <t>footer.tagline</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
+      <c r="B150" t="inlineStr">
         <is>
           <t>footer</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
+      <c r="C150" t="inlineStr">
         <is>
           <t>Footer bottom-right tagline</t>
         </is>
       </c>
-      <c r="D137" t="inlineStr">
+      <c r="D150" t="inlineStr">
         <is>
           <t>Design the business before you build the software.</t>
         </is>

</xml_diff>